<commit_message>
Confere a matriz com d1_pib_vab e adiciona PIB real e bioeconomia à evolução
- Conferência: QLs e EST-02 de 2021, participações de MT e vínculos
  batem com d1_pib_vab.csv; registrada em Fontes e Notas.
- Página: crescimento real do PIB (2010 = 100) contra MT, composição do
  VAB com administração pública e bioeconomia (R$ de 2024) empilhada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLDtP5x9bnGnFC43EPUEKq
</commit_message>
<xml_diff>
--- a/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
+++ b/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
@@ -295,7 +295,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="338">
   <si>
     <t xml:space="preserve">MATRIZ SWOT DO PERFIL ECONÔMICO-PRODUTIVO SETORIAL MUNICIPAL (PESM) — PANTANAL NORTE</t>
   </si>
@@ -910,6 +910,21 @@
   </si>
   <si>
     <t xml:space="preserve">Os 16 grupos da base tratada aproximam as seções CNAE; o HHI é comparável entre municípios e MT porque usa o mesmo recorte.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conferência</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021 / 2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d1_pib_vab.csv (IBGE – PIB dos Municípios)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QLs (AGR-01, IND-01, CS-01) e EST-02 de 2021 recalculados com lq_agro, lq_ind, lq_serv e sh_adespss_va; participações setoriais de MT; vinculos_31dez 2023 comparado com a RAIS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferença máxima menor que 0,001 nos QLs e no EST-02; participações de MT idênticas às da aba Ranking Locacional; vínculos idênticos. O VAB setorial da base também termina em 2021, então a LIMITAÇÃO acima continua valendo.</t>
   </si>
   <si>
     <t xml:space="preserve">PARÂMETROS</t>
@@ -2503,7 +2518,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="B2" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Indicadores (F-W)'!$A$4:$AM$4,0),"")</f>
@@ -2512,7 +2527,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="B3" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Fatores Externos (O-A)'!$A$4:$R$4,0),"")</f>
@@ -2524,7 +2539,7 @@
         <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>102</v>
@@ -2533,16 +2548,16 @@
         <v>31</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>59</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>67</v>
@@ -2551,16 +2566,16 @@
         <v>33</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3364,12 +3379,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4762,7 +4777,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -4808,12 +4823,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6206,7 +6221,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -6252,12 +6267,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7650,7 +7665,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -7696,12 +7711,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9094,7 +9109,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -9140,12 +9155,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10538,7 +10553,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -10584,12 +10599,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11982,7 +11997,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -12028,12 +12043,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13426,7 +13441,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -13472,12 +13487,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14870,7 +14885,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -14916,12 +14931,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16314,7 +16329,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -17181,12 +17196,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18579,7 +18594,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -18625,12 +18640,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20023,7 +20038,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -20069,12 +20084,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21467,7 +21482,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -21513,12 +21528,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22911,7 +22926,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -28353,7 +28368,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -28724,6 +28739,23 @@
       </c>
       <c r="E34" s="58" t="s">
         <v>204</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="58" t="s">
+        <v>205</v>
+      </c>
+      <c r="B35" s="58" t="s">
+        <v>206</v>
+      </c>
+      <c r="C35" s="58" t="s">
+        <v>207</v>
+      </c>
+      <c r="D35" s="58" t="s">
+        <v>208</v>
+      </c>
+      <c r="E35" s="58" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -28758,23 +28790,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="47" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="B3" s="63" t="n">
         <v>0.1</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B4" s="64" t="n">
         <v>2</v>
@@ -28782,18 +28814,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="40" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="B5" s="65" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28920,12 +28952,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28933,40 +28965,40 @@
         <v>59</v>
       </c>
       <c r="B4" s="66" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="C4" s="66" t="s">
         <v>60</v>
       </c>
       <c r="D4" s="66" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="E4" s="66" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="F4" s="66" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="G4" s="66" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="H4" s="66" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="I4" s="66" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="J4" s="66" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="K4" s="66" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="L4" s="66" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="M4" s="66" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="N4" s="66" t="s">
         <v>46</v>
@@ -29036,79 +29068,79 @@
       <c r="L5" s="66"/>
       <c r="M5" s="66"/>
       <c r="N5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="O5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="P5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="Q5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="R5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="S5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="T5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="U5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="V5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="W5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="X5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="Y5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="Z5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="AA5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AB5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="AC5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AD5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="AE5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AF5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="AG5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AH5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="AI5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AJ5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="AK5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AL5" s="67" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="AM5" s="67" t="s">
         <v>102</v>
@@ -29116,28 +29148,28 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="68" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B6" s="69" t="s">
         <v>74</v>
       </c>
       <c r="C6" s="69" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="D6" s="68" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F6" s="69" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="G6" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="I6" s="71" t="n">
         <v>1</v>
@@ -29256,22 +29288,22 @@
         <v>74</v>
       </c>
       <c r="C7" s="69" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="D7" s="68" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F7" s="69" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="G7" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I7" s="71" t="n">
         <v>5602.9</v>
@@ -29386,22 +29418,22 @@
         <v>74</v>
       </c>
       <c r="C8" s="69" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="D8" s="68" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F8" s="69" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="G8" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="I8" s="71" t="n">
         <v>3.79</v>
@@ -29516,20 +29548,20 @@
         <v>74</v>
       </c>
       <c r="C9" s="69" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="D9" s="68" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F9" s="69" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="G9" s="70"/>
       <c r="H9" s="70" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="I9" s="71"/>
       <c r="J9" s="71"/>
@@ -29616,20 +29648,20 @@
         <v>74</v>
       </c>
       <c r="C10" s="69" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="D10" s="68" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="G10" s="70"/>
       <c r="H10" s="70" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I10" s="71"/>
       <c r="J10" s="71"/>
@@ -29710,28 +29742,28 @@
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="75" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="B11" s="76" t="s">
         <v>76</v>
       </c>
       <c r="C11" s="76" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D11" s="75" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F11" s="76" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="G11" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H11" s="70" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="I11" s="71" t="n">
         <v>1</v>
@@ -29850,22 +29882,22 @@
         <v>76</v>
       </c>
       <c r="C12" s="76" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="D12" s="75" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F12" s="76" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="G12" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="I12" s="71" t="n">
         <v>36.92</v>
@@ -29980,22 +30012,22 @@
         <v>76</v>
       </c>
       <c r="C13" s="76" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D13" s="75" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F13" s="76" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="G13" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I13" s="71" t="n">
         <v>2956.72</v>
@@ -30104,28 +30136,28 @@
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="77" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="B14" s="78" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C14" s="78" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D14" s="77" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F14" s="78" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="G14" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="I14" s="71" t="n">
         <v>1</v>
@@ -30241,25 +30273,25 @@
         <v>194</v>
       </c>
       <c r="B15" s="78" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C15" s="78" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="D15" s="77" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F15" s="78" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="G15" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="I15" s="71" t="n">
         <v>38.11</v>
@@ -30371,25 +30403,25 @@
         <v>158</v>
       </c>
       <c r="B16" s="78" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C16" s="78" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D16" s="77" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E16" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F16" s="78" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="G16" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I16" s="71" t="n">
         <v>33.22</v>
@@ -30501,25 +30533,25 @@
         <v>142</v>
       </c>
       <c r="B17" s="80" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C17" s="80" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D17" s="79" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F17" s="80" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="G17" s="70" t="n">
         <v>2023</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I17" s="71" t="n">
         <v>74620.05</v>
@@ -30631,25 +30663,25 @@
         <v>138</v>
       </c>
       <c r="B18" s="80" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C18" s="80" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D18" s="79" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E18" s="70" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="F18" s="80" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="G18" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="I18" s="71" t="n">
         <v>11.89</v>
@@ -30761,25 +30793,25 @@
         <v>199</v>
       </c>
       <c r="B19" s="80" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C19" s="80" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="D19" s="79" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="E19" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F19" s="80" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="G19" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I19" s="71" t="n">
         <v>31.51</v>
@@ -30891,25 +30923,25 @@
         <v>202</v>
       </c>
       <c r="B20" s="80" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C20" s="80" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D20" s="79" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="E20" s="70" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="F20" s="80" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="G20" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I20" s="83" t="n">
         <v>0.1254</v>
@@ -31021,23 +31053,23 @@
         <v>160</v>
       </c>
       <c r="B21" s="80" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C21" s="80" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="D21" s="79" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E21" s="70" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F21" s="80" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="G21" s="70"/>
       <c r="H21" s="70" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="I21" s="71"/>
       <c r="J21" s="71"/>
@@ -31118,7 +31150,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="33" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -31200,12 +31232,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31216,13 +31248,13 @@
         <v>67</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="D4" s="84" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="84" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="F4" s="84" t="s">
         <v>46</v>
@@ -31266,24 +31298,24 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C6" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="F6" s="70" t="n">
         <v>1</v>
@@ -31327,19 +31359,19 @@
     </row>
     <row r="7" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C7" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="F7" s="70" t="n">
         <v>3</v>
@@ -31383,19 +31415,19 @@
     </row>
     <row r="8" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="F8" s="70" t="n">
         <v>3</v>
@@ -31439,19 +31471,19 @@
     </row>
     <row r="9" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C9" s="28" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="F9" s="70" t="n">
         <v>0</v>
@@ -31495,19 +31527,19 @@
     </row>
     <row r="10" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="F10" s="70" t="n">
         <v>1</v>
@@ -31551,19 +31583,19 @@
     </row>
     <row r="11" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="F11" s="70" t="n">
         <v>2</v>
@@ -31607,19 +31639,19 @@
     </row>
     <row r="12" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="85" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B12" s="85" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C12" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D12" s="86" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="E12" s="86" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="F12" s="70" t="n">
         <v>3</v>
@@ -31663,19 +31695,19 @@
     </row>
     <row r="13" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="85" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="B13" s="85" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C13" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D13" s="86" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="E13" s="86" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F13" s="70" t="n">
         <v>2</v>
@@ -31719,19 +31751,19 @@
     </row>
     <row r="14" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="85" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B14" s="85" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C14" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D14" s="86" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E14" s="86" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="F14" s="70" t="n">
         <v>2</v>
@@ -31775,19 +31807,19 @@
     </row>
     <row r="15" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="85" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B15" s="85" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C15" s="86" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D15" s="86" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="E15" s="86" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="F15" s="70" t="n">
         <v>1</v>
@@ -31831,19 +31863,19 @@
     </row>
     <row r="16" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="85" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B16" s="85" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C16" s="86" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="D16" s="86" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="E16" s="86" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="F16" s="70" t="n">
         <v>3</v>
@@ -31887,7 +31919,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Preenche EST-05 (autonomia fiscal 2022) e adiciona a série à página
- EST-05 com d6_financas.csv: receita própria ÷ receita total, 2022 (último
  ano com os 13 municípios); MT = soma dos 141 municípios (18,24%).
  Diferença de denominador (total x corrente) registrada na planilha.
- Página: gráfico de autonomia fiscal 2013-2023 contra MT; cobertura 14/16.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLDtP5x9bnGnFC43EPUEKq
</commit_message>
<xml_diff>
--- a/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
+++ b/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
@@ -206,6 +206,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="G21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">2022: último ano com os 13 municípios (2023 não tem Santo Antônio do Leverger). Fonte: d6_financas.csv (Siconfi/FINBRA), coluna autonomia_fiscal_pct = receita própria ÷ receita TOTAL. Aproxima receita própria ÷ receita corrente; como as receitas de capital são pequenas, a diferença tende a ser pequena, mas o denominador não é o mesmo.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="I7" authorId="0">
       <text>
         <r>
@@ -227,6 +239,18 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">MT: 31.654.882 cab. (2019) → 32.853.368 cab. (2024) = +3,79%.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">MT = Σ receita própria ÷ Σ receita total dos 141 municípios em 2022 (não é o governo estadual).</t>
         </r>
       </text>
     </comment>
@@ -295,7 +319,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="342">
   <si>
     <t xml:space="preserve">MATRIZ SWOT DO PERFIL ECONÔMICO-PRODUTIVO SETORIAL MUNICIPAL (PESM) — PANTANAL NORTE</t>
   </si>
@@ -639,7 +663,7 @@
     <t xml:space="preserve">⚠ RANKING SWOT — COBERTURA MÍNIMA ATINGIDA; NOTAS EXTERNAS A VALIDAR</t>
   </si>
   <si>
-    <t xml:space="preserve">A regra de 75% de cobertura foi atingida em 25/09/2026: 13 de 16 indicadores internos com dado e 11 de 11 fatores externos pontuados. As notas externas ainda são preliminares (uma rodada, pesquisa web-based) e precisam de consenso da equipe antes de uso em relatório.</t>
+    <t xml:space="preserve">A regra de 75% de cobertura foi atingida em 25/09/2026: 14 de 16 indicadores internos com dado e 11 de 11 fatores externos pontuados. As notas externas ainda são preliminares (uma rodada, pesquisa web-based) e precisam de consenso da equipe antes de uso em relatório.</t>
   </si>
   <si>
     <t xml:space="preserve">Indicadores com dado</t>
@@ -744,7 +768,7 @@
     <t xml:space="preserve">O VAB setorial de 2022–2023 já foi divulgado pelo IBGE (dez/2025), mas não estava acessível no ambiente em que esta planilha foi preenchida. Os QLs e o EST-02 usam 2021 e devem ser atualizados pela Tabela 5938 do SIDRA (variáveis de VAB, anos 2022–2023). O PIB per capita (EST-01) já está em 2023.</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDENTES (3 indicadores)</t>
+    <t xml:space="preserve">PENDENTES (2 indicadores)</t>
   </si>
   <si>
     <t xml:space="preserve">AGR-05</t>
@@ -780,7 +804,7 @@
     <t xml:space="preserve">EST-05</t>
   </si>
   <si>
-    <t xml:space="preserve">Siconfi/STN – DCA Anexo I-C (receitas próprias e receita corrente)</t>
+    <t xml:space="preserve">Preenchido em 25/09/2026 com d6_financas.csv (ver bloco "BASES TRATADAS" abaixo).</t>
   </si>
   <si>
     <t xml:space="preserve">RODADA DE 25/09/2026 — FATORES EXTERNOS (O-A)</t>
@@ -798,7 +822,7 @@
     <t xml:space="preserve">Indicadores internos pendentes</t>
   </si>
   <si>
-    <t xml:space="preserve">Pendentes: AGR-04 (Censo Agro 2017, fora do catálogo), AGR-05 (a base só tem diversificação entre lavoura, pecuária, extrativismo e pesca) e EST-05 (depende de d6_financas.csv, ainda não enviado).</t>
+    <t xml:space="preserve">Pendentes: AGR-04 (Censo Agro 2017, fora do catálogo) e AGR-05 (a base só tem diversificação entre lavoura, pecuária, extrativismo e pesca).</t>
   </si>
   <si>
     <t xml:space="preserve">RODADA DE 25/09/2026 — BASES TRATADAS (CATALOGO_BASES_TRATADAS, dimensão D1_PESM)</t>
@@ -925,6 +949,18 @@
   </si>
   <si>
     <t xml:space="preserve">Diferença máxima menor que 0,001 nos QLs e no EST-02; participações de MT idênticas às da aba Ranking Locacional; vínculos idênticos. O VAB setorial da base também termina em 2021, então a LIMITAÇÃO acima continua valendo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d6_financas.csv (Siconfi/FINBRA), coluna autonomia_fiscal_pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receita própria ÷ receita total × 100 (a base não traz a receita corrente). Ref. MT = Σ receita própria ÷ Σ receita total dos 141 municípios = 18.24%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O cálculo com receita_propria_real ÷ receita_total_real reproduz a coluna (diferença &lt; 0,01 p.p.). Denominador diferente do previsto (receita total em vez de corrente): tratar como aproximação.</t>
   </si>
   <si>
     <t xml:space="preserve">PARÂMETROS</t>
@@ -2518,7 +2554,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="B2" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Indicadores (F-W)'!$A$4:$AM$4,0),"")</f>
@@ -2527,7 +2563,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B3" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Fatores Externos (O-A)'!$A$4:$R$4,0),"")</f>
@@ -2539,7 +2575,7 @@
         <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>102</v>
@@ -2548,16 +2584,16 @@
         <v>31</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>59</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>67</v>
@@ -2566,16 +2602,16 @@
         <v>33</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3331,11 +3367,11 @@
       </c>
       <c r="C21" s="1" t="str">
         <f aca="false">IF($B$2="","",INDEX('Indicadores (F-W)'!$A21:$AM21,1,$B$2+1))</f>
-        <v/>
+        <v>Neutro</v>
       </c>
       <c r="D21" s="88" t="n">
         <f aca="false">IF($B$2="","",INDEX('Indicadores (F-W)'!$A21:$AM21,1,$B$2))</f>
-        <v>0</v>
+        <v>17.68</v>
       </c>
       <c r="E21" s="1" t="str">
         <f aca="false">IF(C21="Força",COUNTIF(C$6:C21,"Força"),"")</f>
@@ -3379,18 +3415,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3414,7 +3450,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 9 item(ns)</v>
+        <v>FRAQUEZAS (W) — 10 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -4226,17 +4262,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(10,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F17" s="19" t="str">
+      <c r="F17" s="19" t="n">
         <f aca="false">IF(G17="","",10)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="G17" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(10,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H17" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H17" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(10,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>6.34</v>
       </c>
       <c r="K17" s="1" t="str">
         <f aca="false">Aux!B17</f>
@@ -4390,19 +4426,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!O21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!N21="","",'Indicadores (F-W)'!N21)</f>
-        <v/>
+        <v>6.34</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4777,7 +4813,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -4823,18 +4859,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 2  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 3  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5834,11 +5870,11 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!Q21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Neutro</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!P21="","",'Indicadores (F-W)'!P21)</f>
-        <v/>
+        <v>17.68</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
@@ -6221,7 +6257,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -6267,18 +6303,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6302,7 +6338,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 9 item(ns)</v>
+        <v>FRAQUEZAS (W) — 10 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -7114,17 +7150,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(10,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F17" s="19" t="str">
+      <c r="F17" s="19" t="n">
         <f aca="false">IF(G17="","",10)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="G17" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(10,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H17" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H17" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(10,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>5.5</v>
       </c>
       <c r="K17" s="1" t="str">
         <f aca="false">Aux!B17</f>
@@ -7278,19 +7314,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!S21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!R21="","",'Indicadores (F-W)'!R21)</f>
-        <v/>
+        <v>5.5</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7665,7 +7701,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -7711,18 +7747,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7746,7 +7782,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 9 item(ns)</v>
+        <v>FRAQUEZAS (W) — 10 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -8558,17 +8594,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(10,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F17" s="19" t="str">
+      <c r="F17" s="19" t="n">
         <f aca="false">IF(G17="","",10)</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="G17" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(10,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H17" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H17" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(10,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>5.76</v>
       </c>
       <c r="K17" s="1" t="str">
         <f aca="false">Aux!B17</f>
@@ -8722,19 +8758,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!U21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!T21="","",'Indicadores (F-W)'!T21)</f>
-        <v/>
+        <v>5.76</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9109,7 +9145,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -9155,18 +9191,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9190,7 +9226,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 5 item(ns)</v>
+        <v>FRAQUEZAS (W) — 6 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -9702,17 +9738,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(6,$N$6:$N$21,0)),"")</f>
         <v>5.88</v>
       </c>
-      <c r="F13" s="19" t="str">
+      <c r="F13" s="19" t="n">
         <f aca="false">IF(G13="","",6)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="G13" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(6,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H13" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H13" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(6,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>11.87</v>
       </c>
       <c r="K13" s="1" t="str">
         <f aca="false">Aux!B13</f>
@@ -10166,19 +10202,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!W21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!V21="","",'Indicadores (F-W)'!V21)</f>
-        <v/>
+        <v>11.87</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>6</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10553,7 +10589,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -10599,18 +10635,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 4  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 4  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10634,7 +10670,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 6 item(ns)</v>
+        <v>FRAQUEZAS (W) — 7 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -11221,17 +11257,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(7,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F14" s="19" t="str">
+      <c r="F14" s="19" t="n">
         <f aca="false">IF(G14="","",7)</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="G14" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(7,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H14" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H14" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(7,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>11.71</v>
       </c>
       <c r="K14" s="1" t="str">
         <f aca="false">Aux!B14</f>
@@ -11610,19 +11646,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!Y21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!X21="","",'Indicadores (F-W)'!X21)</f>
-        <v/>
+        <v>11.71</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>7</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11997,7 +12033,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -12043,18 +12079,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 3  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 3  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12078,7 +12114,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 8 item(ns)</v>
+        <v>FRAQUEZAS (W) — 9 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -12815,17 +12851,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(9,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F16" s="19" t="str">
+      <c r="F16" s="19" t="n">
         <f aca="false">IF(G16="","",9)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="G16" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(9,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H16" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H16" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(9,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>7.14</v>
       </c>
       <c r="K16" s="1" t="str">
         <f aca="false">Aux!B16</f>
@@ -13054,19 +13090,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!AA21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!Z21="","",'Indicadores (F-W)'!Z21)</f>
-        <v/>
+        <v>7.14</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>9</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13441,7 +13477,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -13487,18 +13523,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 4  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 4  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13522,7 +13558,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 7 item(ns)</v>
+        <v>FRAQUEZAS (W) — 8 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -14184,17 +14220,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(8,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F15" s="19" t="str">
+      <c r="F15" s="19" t="n">
         <f aca="false">IF(G15="","",8)</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="G15" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(8,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H15" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H15" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(8,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>14.35</v>
       </c>
       <c r="K15" s="1" t="str">
         <f aca="false">Aux!B15</f>
@@ -14498,19 +14534,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!AC21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!AB21="","",'Indicadores (F-W)'!AB21)</f>
-        <v/>
+        <v>14.35</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>8</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14885,7 +14921,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -14931,18 +14967,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 2  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 2  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14966,7 +15002,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 7 item(ns)</v>
+        <v>FRAQUEZAS (W) — 8 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -15628,17 +15664,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(8,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F15" s="19" t="str">
+      <c r="F15" s="19" t="n">
         <f aca="false">IF(G15="","",8)</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="G15" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(8,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H15" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H15" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(8,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>5.15</v>
       </c>
       <c r="K15" s="1" t="str">
         <f aca="false">Aux!B15</f>
@@ -15942,19 +15978,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!AE21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!AD21="","",'Indicadores (F-W)'!AD21)</f>
-        <v/>
+        <v>5.15</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>8</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16329,7 +16365,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -16386,7 +16422,7 @@
       <c r="D3" s="8"/>
       <c r="F3" s="9" t="str">
         <f aca="false">"Indicadores: "&amp;COUNTIF(Aux!$C$6:$C$21,"Neutro")&amp;" neutros | "&amp;(COUNTA(Aux!$A$6:$A$21)-COUNTIF(Aux!$C$6:$C$21,"Força")-COUNTIF(Aux!$C$6:$C$21,"Fraqueza")-COUNTIF(Aux!$C$6:$C$21,"Neutro"))&amp;" sem dado"</f>
-        <v>Indicadores: 2 neutros | 3 sem dado</v>
+        <v>Indicadores: 3 neutros | 2 sem dado</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17196,18 +17232,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 2  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 2  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17231,7 +17267,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 10 item(ns)</v>
+        <v>FRAQUEZAS (W) — 11 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -18090,17 +18126,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(11,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F18" s="19" t="str">
+      <c r="F18" s="19" t="n">
         <f aca="false">IF(G18="","",11)</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="G18" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(11,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H18" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H18" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(11,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>9.51</v>
       </c>
       <c r="K18" s="1" t="str">
         <f aca="false">Aux!B18</f>
@@ -18207,19 +18243,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!AG21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!AF21="","",'Indicadores (F-W)'!AF21)</f>
-        <v/>
+        <v>9.51</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18594,7 +18630,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -18640,18 +18676,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 2  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 2  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18675,7 +18711,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 8 item(ns)</v>
+        <v>FRAQUEZAS (W) — 9 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -19412,17 +19448,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(9,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F16" s="19" t="str">
+      <c r="F16" s="19" t="n">
         <f aca="false">IF(G16="","",9)</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="G16" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(9,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H16" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H16" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(9,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>6.54</v>
       </c>
       <c r="K16" s="1" t="str">
         <f aca="false">Aux!B16</f>
@@ -19651,19 +19687,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!AI21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!AH21="","",'Indicadores (F-W)'!AH21)</f>
-        <v/>
+        <v>6.54</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>9</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20038,7 +20074,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -20084,18 +20120,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 7  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 7  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20113,7 +20149,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="11" t="str">
         <f aca="false">"FORÇAS (S) — "&amp;COUNTIF($L$6:$L$21,"Força")&amp;" item(ns)"</f>
-        <v>FORÇAS (S) — 3 item(ns)</v>
+        <v>FORÇAS (S) — 4 item(ns)</v>
       </c>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
@@ -20469,17 +20505,17 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15"/>
-      <c r="B11" s="16" t="str">
+      <c r="B11" s="16" t="n">
         <f aca="false">IF(C11="","",4)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="C11" s="17" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(4,$N$6:$N$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D11" s="18" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="D11" s="18" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(4,$N$6:$N$21,0)),"")</f>
-        <v/>
+        <v>21.61</v>
       </c>
       <c r="F11" s="19" t="str">
         <f aca="false">IF(G11="","",4)</f>
@@ -21095,15 +21131,15 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!AK21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Força</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!AJ21="","",'Indicadores (F-W)'!AJ21)</f>
-        <v/>
-      </c>
-      <c r="N21" s="1" t="str">
+        <v>21.61</v>
+      </c>
+      <c r="N21" s="1" t="n">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="O21" s="1" t="str">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
@@ -21482,7 +21518,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -21528,18 +21564,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="92" t="str">
         <f aca="false">"Indicadores internos com dado: "&amp;(COUNTA(L6:L21)-COUNTBLANK(L6:L21))&amp;" de 16  |  Neutros: "&amp;COUNTIF(L6:L21,"Neutro")&amp;"  |  Fatores externos pontuados: "&amp;COUNT(S6:S16)&amp;" de 11"</f>
-        <v>Indicadores internos com dado: 13 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
+        <v>Indicadores internos com dado: 14 de 16  |  Neutros: 1  |  Fatores externos pontuados: 11 de 11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21563,7 +21599,7 @@
       <c r="D6" s="11"/>
       <c r="F6" s="12" t="str">
         <f aca="false">"FRAQUEZAS (W) — "&amp;COUNTIF($L$6:$L$21,"Fraqueza")&amp;" item(ns)"</f>
-        <v>FRAQUEZAS (W) — 10 item(ns)</v>
+        <v>FRAQUEZAS (W) — 11 item(ns)</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
@@ -22422,17 +22458,17 @@
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(11,$N$6:$N$21,0)),"")</f>
         <v/>
       </c>
-      <c r="F18" s="19" t="str">
+      <c r="F18" s="19" t="n">
         <f aca="false">IF(G18="","",11)</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="G18" s="20" t="str">
         <f aca="false">IFERROR(INDEX($K$6:$K$21,MATCH(11,$O$6:$O$21,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H18" s="21" t="str">
+        <v>[Estrutura Econômica e Fiscal] EST-05 – Receitas próprias / receita corrente (%)</v>
+      </c>
+      <c r="H18" s="21" t="n">
         <f aca="false">IFERROR(INDEX($M$6:$M$21,MATCH(11,$O$6:$O$21,0)),"")</f>
-        <v/>
+        <v>9.96</v>
       </c>
       <c r="K18" s="1" t="str">
         <f aca="false">Aux!B18</f>
@@ -22539,19 +22575,19 @@
       </c>
       <c r="L21" s="1" t="str">
         <f aca="false">'Indicadores (F-W)'!AM21</f>
-        <v/>
-      </c>
-      <c r="M21" s="1" t="str">
+        <v>Fraqueza</v>
+      </c>
+      <c r="M21" s="88" t="n">
         <f aca="false">IF('Indicadores (F-W)'!AL21="","",'Indicadores (F-W)'!AL21)</f>
-        <v/>
+        <v>9.96</v>
       </c>
       <c r="N21" s="1" t="str">
         <f aca="false">IF(L21="Força",COUNTIF(L$6:L21,"Força"),"")</f>
         <v/>
       </c>
-      <c r="O21" s="1" t="str">
+      <c r="O21" s="1" t="n">
         <f aca="false">IF(L21="Fraqueza",COUNTIF(L$6:L21,"Fraqueza"),"")</f>
-        <v/>
+        <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22926,7 +22962,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -23012,7 +23048,7 @@
       </c>
       <c r="C4" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!O$6:O$21,"Fraqueza")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D4" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!O$6:O$21,"Neutro")</f>
@@ -23020,11 +23056,11 @@
       </c>
       <c r="E4" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!N$6:N$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" s="36" t="n">
         <f aca="false">B4-C4</f>
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="G4" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!F$6:F$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23053,11 +23089,11 @@
       </c>
       <c r="D5" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!Q$6:Q$21,"Neutro")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!P$6:P$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="36" t="n">
         <f aca="false">B5-C5</f>
@@ -23086,7 +23122,7 @@
       </c>
       <c r="C6" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!S$6:S$21,"Fraqueza")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!S$6:S$21,"Neutro")</f>
@@ -23094,11 +23130,11 @@
       </c>
       <c r="E6" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!R$6:R$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" s="36" t="n">
         <f aca="false">B6-C6</f>
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="G6" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!H$6:H$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23123,7 +23159,7 @@
       </c>
       <c r="C7" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!U$6:U$21,"Fraqueza")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!U$6:U$21,"Neutro")</f>
@@ -23131,11 +23167,11 @@
       </c>
       <c r="E7" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!T$6:T$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" s="36" t="n">
         <f aca="false">B7-C7</f>
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="G7" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!I$6:I$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23160,7 +23196,7 @@
       </c>
       <c r="C8" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!W$6:W$21,"Fraqueza")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D8" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!W$6:W$21,"Neutro")</f>
@@ -23168,11 +23204,11 @@
       </c>
       <c r="E8" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!V$6:V$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" s="36" t="n">
         <f aca="false">B8-C8</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!J$6:J$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23197,7 +23233,7 @@
       </c>
       <c r="C9" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!Y$6:Y$21,"Fraqueza")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D9" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!Y$6:Y$21,"Neutro")</f>
@@ -23205,11 +23241,11 @@
       </c>
       <c r="E9" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!X$6:X$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" s="36" t="n">
         <f aca="false">B9-C9</f>
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G9" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!K$6:K$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23234,7 +23270,7 @@
       </c>
       <c r="C10" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AA$6:AA$21,"Fraqueza")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D10" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AA$6:AA$21,"Neutro")</f>
@@ -23242,11 +23278,11 @@
       </c>
       <c r="E10" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!Z$6:Z$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" s="36" t="n">
         <f aca="false">B10-C10</f>
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="G10" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!L$6:L$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23271,7 +23307,7 @@
       </c>
       <c r="C11" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AC$6:AC$21,"Fraqueza")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D11" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AC$6:AC$21,"Neutro")</f>
@@ -23279,11 +23315,11 @@
       </c>
       <c r="E11" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!AB$6:AB$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" s="36" t="n">
         <f aca="false">B11-C11</f>
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="G11" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!M$6:M$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23308,7 +23344,7 @@
       </c>
       <c r="C12" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AE$6:AE$21,"Fraqueza")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D12" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AE$6:AE$21,"Neutro")</f>
@@ -23316,11 +23352,11 @@
       </c>
       <c r="E12" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!AD$6:AD$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" s="36" t="n">
         <f aca="false">B12-C12</f>
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G12" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!N$6:N$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23345,7 +23381,7 @@
       </c>
       <c r="C13" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AG$6:AG$21,"Fraqueza")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D13" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AG$6:AG$21,"Neutro")</f>
@@ -23353,11 +23389,11 @@
       </c>
       <c r="E13" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!AF$6:AF$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" s="36" t="n">
         <f aca="false">B13-C13</f>
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G13" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!O$6:O$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23382,7 +23418,7 @@
       </c>
       <c r="C14" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AI$6:AI$21,"Fraqueza")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D14" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AI$6:AI$21,"Neutro")</f>
@@ -23390,11 +23426,11 @@
       </c>
       <c r="E14" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!AH$6:AH$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" s="36" t="n">
         <f aca="false">B14-C14</f>
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="G14" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!P$6:P$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23415,7 +23451,7 @@
       </c>
       <c r="B15" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AK$6:AK$21,"Força")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AK$6:AK$21,"Fraqueza")</f>
@@ -23427,11 +23463,11 @@
       </c>
       <c r="E15" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!AJ$6:AJ$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" s="36" t="n">
         <f aca="false">B15-C15</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!Q$6:Q$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23456,7 +23492,7 @@
       </c>
       <c r="C16" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AM$6:AM$21,"Fraqueza")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D16" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!AM$6:AM$21,"Neutro")</f>
@@ -23464,11 +23500,11 @@
       </c>
       <c r="E16" s="36" t="n">
         <f aca="false">COUNTBLANK('Indicadores (F-W)'!AL$6:AL$21)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" s="36" t="n">
         <f aca="false">B16-C16</f>
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="G16" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Oportunidade",'Fatores Externos (O-A)'!R$6:R$16,"&gt;="&amp;Parâmetros!$B$5)</f>
@@ -23972,23 +24008,23 @@
       </c>
       <c r="C36" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!$N21:$AM21,"Força")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!$N21:$AM21,"Neutro")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="36" t="n">
         <f aca="false">COUNTIF('Indicadores (F-W)'!$N21:$AM21,"Fraqueza")</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F36" s="36" t="n">
         <f aca="false">13-C36-D36-E36</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G36" s="36" t="str">
         <f aca="false">IF(C36+D36+E36=0,"sem dados",IF(C36&gt;=13/2,"Força regional",IF(E36&gt;=13/2,"Fraqueza regional","Heterogêneo")))</f>
-        <v>sem dados</v>
+        <v>Fraqueza regional</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27123,19 +27159,19 @@
       </c>
       <c r="C5" s="53" t="n">
         <f aca="false">Painel!C4</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="53" t="n">
         <f aca="false">16-Painel!E4</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="54" t="n">
         <f aca="false">D5/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F5" s="55" t="n">
         <f aca="false">IF(D5=0,"",(B5-C5)/D5)</f>
-        <v>-0.461538461538462</v>
+        <v>-0.5</v>
       </c>
       <c r="G5" s="53" t="n">
         <f aca="false">Painel!G4</f>
@@ -27159,7 +27195,7 @@
       </c>
       <c r="L5" s="56" t="n">
         <f aca="false">IF(F5="","",IF(K5="",F5,(F5+K5)/2))</f>
-        <v>-0.276223776223776</v>
+        <v>-0.295454545454545</v>
       </c>
       <c r="M5" s="46" t="n">
         <f aca="false">IF(L5="","",RANK(L5,$L$5:$L$17,0))</f>
@@ -27171,7 +27207,7 @@
       </c>
       <c r="T5" s="1" t="n">
         <f aca="false">IF(L5="",-9,L5)-ROW()*0.000000001</f>
-        <v>-0.276223781223776</v>
+        <v>-0.295454550454546</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27188,15 +27224,15 @@
       </c>
       <c r="D6" s="53" t="n">
         <f aca="false">16-Painel!E5</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E6" s="54" t="n">
         <f aca="false">D6/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F6" s="55" t="n">
         <f aca="false">IF(D6=0,"",(B6-C6)/D6)</f>
-        <v>-0.384615384615385</v>
+        <v>-0.357142857142857</v>
       </c>
       <c r="G6" s="53" t="n">
         <f aca="false">Painel!G5</f>
@@ -27220,11 +27256,11 @@
       </c>
       <c r="L6" s="56" t="n">
         <f aca="false">IF(F6="","",IF(K6="",F6,(F6+K6)/2))</f>
-        <v>-0.101398601398601</v>
+        <v>-0.0876623376623377</v>
       </c>
       <c r="M6" s="46" t="n">
         <f aca="false">IF(L6="","",RANK(L6,$L$5:$L$17,0))</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N6" s="49" t="str">
         <f aca="false">IF(AND(E6&gt;=0.75,J6&gt;=0.75),"Consolidado","PROVISÓRIO")</f>
@@ -27232,7 +27268,7 @@
       </c>
       <c r="T6" s="1" t="n">
         <f aca="false">IF(L6="",-9,L6)-ROW()*0.000000001</f>
-        <v>-0.101398607398601</v>
+        <v>-0.0876623436623377</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27245,19 +27281,19 @@
       </c>
       <c r="C7" s="53" t="n">
         <f aca="false">Painel!C6</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="53" t="n">
         <f aca="false">16-Painel!E6</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" s="54" t="n">
         <f aca="false">D7/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F7" s="55" t="n">
         <f aca="false">IF(D7=0,"",(B7-C7)/D7)</f>
-        <v>-0.461538461538462</v>
+        <v>-0.5</v>
       </c>
       <c r="G7" s="53" t="n">
         <f aca="false">Painel!G6</f>
@@ -27281,7 +27317,7 @@
       </c>
       <c r="L7" s="56" t="n">
         <f aca="false">IF(F7="","",IF(K7="",F7,(F7+K7)/2))</f>
-        <v>-0.276223776223776</v>
+        <v>-0.295454545454545</v>
       </c>
       <c r="M7" s="46" t="n">
         <f aca="false">IF(L7="","",RANK(L7,$L$5:$L$17,0))</f>
@@ -27293,7 +27329,7 @@
       </c>
       <c r="T7" s="1" t="n">
         <f aca="false">IF(L7="",-9,L7)-ROW()*0.000000001</f>
-        <v>-0.276223783223776</v>
+        <v>-0.295454552454546</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27306,19 +27342,19 @@
       </c>
       <c r="C8" s="53" t="n">
         <f aca="false">Painel!C7</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D8" s="53" t="n">
         <f aca="false">16-Painel!E7</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E8" s="54" t="n">
         <f aca="false">D8/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F8" s="55" t="n">
         <f aca="false">IF(D8=0,"",(B8-C8)/D8)</f>
-        <v>-0.461538461538462</v>
+        <v>-0.5</v>
       </c>
       <c r="G8" s="53" t="n">
         <f aca="false">Painel!G7</f>
@@ -27342,7 +27378,7 @@
       </c>
       <c r="L8" s="56" t="n">
         <f aca="false">IF(F8="","",IF(K8="",F8,(F8+K8)/2))</f>
-        <v>-0.276223776223776</v>
+        <v>-0.295454545454545</v>
       </c>
       <c r="M8" s="46" t="n">
         <f aca="false">IF(L8="","",RANK(L8,$L$5:$L$17,0))</f>
@@ -27354,7 +27390,7 @@
       </c>
       <c r="T8" s="1" t="n">
         <f aca="false">IF(L8="",-9,L8)-ROW()*0.000000001</f>
-        <v>-0.276223784223776</v>
+        <v>-0.295454553454545</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27367,19 +27403,19 @@
       </c>
       <c r="C9" s="53" t="n">
         <f aca="false">Painel!C8</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" s="53" t="n">
         <f aca="false">16-Painel!E8</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="54" t="n">
         <f aca="false">D9/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F9" s="55" t="n">
         <f aca="false">IF(D9=0,"",(B9-C9)/D9)</f>
-        <v>0.153846153846154</v>
+        <v>0.0714285714285714</v>
       </c>
       <c r="G9" s="53" t="n">
         <f aca="false">Painel!G8</f>
@@ -27403,7 +27439,7 @@
       </c>
       <c r="L9" s="56" t="n">
         <f aca="false">IF(F9="","",IF(K9="",F9,(F9+K9)/2))</f>
-        <v>0.0769230769230769</v>
+        <v>0.0357142857142857</v>
       </c>
       <c r="M9" s="46" t="n">
         <f aca="false">IF(L9="","",RANK(L9,$L$5:$L$17,0))</f>
@@ -27415,7 +27451,7 @@
       </c>
       <c r="T9" s="1" t="n">
         <f aca="false">IF(L9="",-9,L9)-ROW()*0.000000001</f>
-        <v>0.0769230679230769</v>
+        <v>0.0357142767142857</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27428,19 +27464,19 @@
       </c>
       <c r="C10" s="53" t="n">
         <f aca="false">Painel!C9</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D10" s="53" t="n">
         <f aca="false">16-Painel!E9</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E10" s="54" t="n">
         <f aca="false">D10/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F10" s="55" t="n">
         <f aca="false">IF(D10=0,"",(B10-C10)/D10)</f>
-        <v>-0.230769230769231</v>
+        <v>-0.285714285714286</v>
       </c>
       <c r="G10" s="53" t="n">
         <f aca="false">Painel!G9</f>
@@ -27464,11 +27500,11 @@
       </c>
       <c r="L10" s="56" t="n">
         <f aca="false">IF(F10="","",IF(K10="",F10,(F10+K10)/2))</f>
-        <v>-0.0699300699300699</v>
+        <v>-0.0974025974025974</v>
       </c>
       <c r="M10" s="46" t="n">
         <f aca="false">IF(L10="","",RANK(L10,$L$5:$L$17,0))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10" s="49" t="str">
         <f aca="false">IF(AND(E10&gt;=0.75,J10&gt;=0.75),"Consolidado","PROVISÓRIO")</f>
@@ -27476,7 +27512,7 @@
       </c>
       <c r="T10" s="1" t="n">
         <f aca="false">IF(L10="",-9,L10)-ROW()*0.000000001</f>
-        <v>-0.0699300799300699</v>
+        <v>-0.0974026074025974</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27489,19 +27525,19 @@
       </c>
       <c r="C11" s="53" t="n">
         <f aca="false">Painel!C10</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D11" s="53" t="n">
         <f aca="false">16-Painel!E10</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" s="54" t="n">
         <f aca="false">D11/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F11" s="55" t="n">
         <f aca="false">IF(D11=0,"",(B11-C11)/D11)</f>
-        <v>-0.461538461538462</v>
+        <v>-0.5</v>
       </c>
       <c r="G11" s="53" t="n">
         <f aca="false">Painel!G10</f>
@@ -27525,7 +27561,7 @@
       </c>
       <c r="L11" s="56" t="n">
         <f aca="false">IF(F11="","",IF(K11="",F11,(F11+K11)/2))</f>
-        <v>-0.276223776223776</v>
+        <v>-0.295454545454545</v>
       </c>
       <c r="M11" s="46" t="n">
         <f aca="false">IF(L11="","",RANK(L11,$L$5:$L$17,0))</f>
@@ -27537,7 +27573,7 @@
       </c>
       <c r="T11" s="1" t="n">
         <f aca="false">IF(L11="",-9,L11)-ROW()*0.000000001</f>
-        <v>-0.276223787223776</v>
+        <v>-0.295454556454546</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27550,19 +27586,19 @@
       </c>
       <c r="C12" s="53" t="n">
         <f aca="false">Painel!C11</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D12" s="53" t="n">
         <f aca="false">16-Painel!E11</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E12" s="54" t="n">
         <f aca="false">D12/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F12" s="55" t="n">
         <f aca="false">IF(D12=0,"",(B12-C12)/D12)</f>
-        <v>-0.384615384615385</v>
+        <v>-0.428571428571429</v>
       </c>
       <c r="G12" s="53" t="n">
         <f aca="false">Painel!G11</f>
@@ -27586,7 +27622,7 @@
       </c>
       <c r="L12" s="56" t="n">
         <f aca="false">IF(F12="","",IF(K12="",F12,(F12+K12)/2))</f>
-        <v>-0.055944055944056</v>
+        <v>-0.0779220779220779</v>
       </c>
       <c r="M12" s="46" t="n">
         <f aca="false">IF(L12="","",RANK(L12,$L$5:$L$17,0))</f>
@@ -27598,7 +27634,7 @@
       </c>
       <c r="T12" s="1" t="n">
         <f aca="false">IF(L12="",-9,L12)-ROW()*0.000000001</f>
-        <v>-0.055944067944056</v>
+        <v>-0.0779220899220779</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27611,19 +27647,19 @@
       </c>
       <c r="C13" s="53" t="n">
         <f aca="false">Painel!C12</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D13" s="53" t="n">
         <f aca="false">16-Painel!E12</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E13" s="54" t="n">
         <f aca="false">D13/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F13" s="55" t="n">
         <f aca="false">IF(D13=0,"",(B13-C13)/D13)</f>
-        <v>-0.230769230769231</v>
+        <v>-0.285714285714286</v>
       </c>
       <c r="G13" s="53" t="n">
         <f aca="false">Painel!G12</f>
@@ -27647,11 +27683,11 @@
       </c>
       <c r="L13" s="56" t="n">
         <f aca="false">IF(F13="","",IF(K13="",F13,(F13+K13)/2))</f>
-        <v>-0.0699300699300699</v>
+        <v>-0.0974025974025974</v>
       </c>
       <c r="M13" s="46" t="n">
         <f aca="false">IF(L13="","",RANK(L13,$L$5:$L$17,0))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N13" s="49" t="str">
         <f aca="false">IF(AND(E13&gt;=0.75,J13&gt;=0.75),"Consolidado","PROVISÓRIO")</f>
@@ -27659,7 +27695,7 @@
       </c>
       <c r="T13" s="1" t="n">
         <f aca="false">IF(L13="",-9,L13)-ROW()*0.000000001</f>
-        <v>-0.0699300829300699</v>
+        <v>-0.0974026104025974</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27672,19 +27708,19 @@
       </c>
       <c r="C14" s="53" t="n">
         <f aca="false">Painel!C13</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D14" s="53" t="n">
         <f aca="false">16-Painel!E13</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E14" s="54" t="n">
         <f aca="false">D14/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F14" s="55" t="n">
         <f aca="false">IF(D14=0,"",(B14-C14)/D14)</f>
-        <v>-0.692307692307692</v>
+        <v>-0.714285714285714</v>
       </c>
       <c r="G14" s="53" t="n">
         <f aca="false">Painel!G13</f>
@@ -27708,7 +27744,7 @@
       </c>
       <c r="L14" s="56" t="n">
         <f aca="false">IF(F14="","",IF(K14="",F14,(F14+K14)/2))</f>
-        <v>-0.346153846153846</v>
+        <v>-0.357142857142857</v>
       </c>
       <c r="M14" s="46" t="n">
         <f aca="false">IF(L14="","",RANK(L14,$L$5:$L$17,0))</f>
@@ -27720,7 +27756,7 @@
       </c>
       <c r="T14" s="1" t="n">
         <f aca="false">IF(L14="",-9,L14)-ROW()*0.000000001</f>
-        <v>-0.346153860153846</v>
+        <v>-0.357142871142857</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27733,19 +27769,19 @@
       </c>
       <c r="C15" s="53" t="n">
         <f aca="false">Painel!C14</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" s="53" t="n">
         <f aca="false">16-Painel!E14</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E15" s="54" t="n">
         <f aca="false">D15/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F15" s="55" t="n">
         <f aca="false">IF(D15=0,"",(B15-C15)/D15)</f>
-        <v>-0.384615384615385</v>
+        <v>-0.428571428571429</v>
       </c>
       <c r="G15" s="53" t="n">
         <f aca="false">Painel!G14</f>
@@ -27769,7 +27805,7 @@
       </c>
       <c r="L15" s="56" t="n">
         <f aca="false">IF(F15="","",IF(K15="",F15,(F15+K15)/2))</f>
-        <v>-0.237762237762238</v>
+        <v>-0.25974025974026</v>
       </c>
       <c r="M15" s="46" t="n">
         <f aca="false">IF(L15="","",RANK(L15,$L$5:$L$17,0))</f>
@@ -27781,7 +27817,7 @@
       </c>
       <c r="T15" s="1" t="n">
         <f aca="false">IF(L15="",-9,L15)-ROW()*0.000000001</f>
-        <v>-0.237762252762238</v>
+        <v>-0.25974027474026</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27790,7 +27826,7 @@
       </c>
       <c r="B16" s="53" t="n">
         <f aca="false">Painel!B15</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C16" s="53" t="n">
         <f aca="false">Painel!C15</f>
@@ -27798,15 +27834,15 @@
       </c>
       <c r="D16" s="53" t="n">
         <f aca="false">16-Painel!E15</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E16" s="54" t="n">
         <f aca="false">D16/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F16" s="55" t="n">
         <f aca="false">IF(D16=0,"",(B16-C16)/D16)</f>
-        <v>0</v>
+        <v>0.0714285714285714</v>
       </c>
       <c r="G16" s="53" t="n">
         <f aca="false">Painel!G15</f>
@@ -27830,7 +27866,7 @@
       </c>
       <c r="L16" s="56" t="n">
         <f aca="false">IF(F16="","",IF(K16="",F16,(F16+K16)/2))</f>
-        <v>0.0909090909090909</v>
+        <v>0.126623376623377</v>
       </c>
       <c r="M16" s="46" t="n">
         <f aca="false">IF(L16="","",RANK(L16,$L$5:$L$17,0))</f>
@@ -27842,7 +27878,7 @@
       </c>
       <c r="T16" s="1" t="n">
         <f aca="false">IF(L16="",-9,L16)-ROW()*0.000000001</f>
-        <v>0.0909090749090909</v>
+        <v>0.126623360623377</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27855,19 +27891,19 @@
       </c>
       <c r="C17" s="53" t="n">
         <f aca="false">Painel!C16</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D17" s="53" t="n">
         <f aca="false">16-Painel!E16</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E17" s="54" t="n">
         <f aca="false">D17/16</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="F17" s="55" t="n">
         <f aca="false">IF(D17=0,"",(B17-C17)/D17)</f>
-        <v>-0.615384615384615</v>
+        <v>-0.642857142857143</v>
       </c>
       <c r="G17" s="53" t="n">
         <f aca="false">Painel!G16</f>
@@ -27891,7 +27927,7 @@
       </c>
       <c r="L17" s="56" t="n">
         <f aca="false">IF(F17="","",IF(K17="",F17,(F17+K17)/2))</f>
-        <v>-0.307692307692308</v>
+        <v>-0.321428571428571</v>
       </c>
       <c r="M17" s="46" t="n">
         <f aca="false">IF(L17="","",RANK(L17,$L$5:$L$17,0))</f>
@@ -27903,7 +27939,7 @@
       </c>
       <c r="T17" s="1" t="n">
         <f aca="false">IF(L17="",-9,L17)-ROW()*0.000000001</f>
-        <v>-0.307692324692308</v>
+        <v>-0.321428588428571</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27942,11 +27978,11 @@
       </c>
       <c r="C22" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,1),$T$5:$T$17,0))</f>
-        <v>0.0909090909090909</v>
+        <v>0.126623376623377</v>
       </c>
       <c r="D22" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,1),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E22" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,1),$T$5:$T$17,0))</f>
@@ -27968,11 +28004,11 @@
       </c>
       <c r="C23" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,2),$T$5:$T$17,0))</f>
-        <v>0.0769230769230769</v>
+        <v>0.0357142857142857</v>
       </c>
       <c r="D23" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,2),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E23" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,2),$T$5:$T$17,0))</f>
@@ -27994,11 +28030,11 @@
       </c>
       <c r="C24" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,3),$T$5:$T$17,0))</f>
-        <v>-0.055944055944056</v>
+        <v>-0.0779220779220779</v>
       </c>
       <c r="D24" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,3),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E24" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,3),$T$5:$T$17,0))</f>
@@ -28016,15 +28052,15 @@
       </c>
       <c r="B25" s="38" t="str">
         <f aca="false">INDEX($A$5:$A$17,MATCH(LARGE($T$5:$T$17,4),$T$5:$T$17,0))</f>
-        <v>Juscimeira</v>
+        <v>Cáceres</v>
       </c>
       <c r="C25" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,4),$T$5:$T$17,0))</f>
-        <v>-0.0699300699300699</v>
+        <v>-0.0876623376623377</v>
       </c>
       <c r="D25" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,4),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E25" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,4),$T$5:$T$17,0))</f>
@@ -28038,19 +28074,19 @@
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="46" t="n">
         <f aca="false">INDEX($M$5:$M$17,MATCH(LARGE($T$5:$T$17,5),$T$5:$T$17,0))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B26" s="38" t="str">
         <f aca="false">INDEX($A$5:$A$17,MATCH(LARGE($T$5:$T$17,5),$T$5:$T$17,0))</f>
-        <v>Nossa Senhora do Livramento</v>
+        <v>Juscimeira</v>
       </c>
       <c r="C26" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,5),$T$5:$T$17,0))</f>
-        <v>-0.0699300699300699</v>
+        <v>-0.0974025974025974</v>
       </c>
       <c r="D26" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,5),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E26" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,5),$T$5:$T$17,0))</f>
@@ -28064,19 +28100,19 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="46" t="n">
         <f aca="false">INDEX($M$5:$M$17,MATCH(LARGE($T$5:$T$17,6),$T$5:$T$17,0))</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27" s="38" t="str">
         <f aca="false">INDEX($A$5:$A$17,MATCH(LARGE($T$5:$T$17,6),$T$5:$T$17,0))</f>
-        <v>Cáceres</v>
+        <v>Nossa Senhora do Livramento</v>
       </c>
       <c r="C27" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,6),$T$5:$T$17,0))</f>
-        <v>-0.101398601398601</v>
+        <v>-0.0974025974025974</v>
       </c>
       <c r="D27" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,6),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E27" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,6),$T$5:$T$17,0))</f>
@@ -28098,11 +28134,11 @@
       </c>
       <c r="C28" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,7),$T$5:$T$17,0))</f>
-        <v>-0.237762237762238</v>
+        <v>-0.25974025974026</v>
       </c>
       <c r="D28" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,7),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E28" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,7),$T$5:$T$17,0))</f>
@@ -28124,11 +28160,11 @@
       </c>
       <c r="C29" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,8),$T$5:$T$17,0))</f>
-        <v>-0.276223776223776</v>
+        <v>-0.295454545454545</v>
       </c>
       <c r="D29" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,8),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E29" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,8),$T$5:$T$17,0))</f>
@@ -28150,11 +28186,11 @@
       </c>
       <c r="C30" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,9),$T$5:$T$17,0))</f>
-        <v>-0.276223776223776</v>
+        <v>-0.295454545454545</v>
       </c>
       <c r="D30" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,9),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E30" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,9),$T$5:$T$17,0))</f>
@@ -28176,11 +28212,11 @@
       </c>
       <c r="C31" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,10),$T$5:$T$17,0))</f>
-        <v>-0.276223776223776</v>
+        <v>-0.295454545454545</v>
       </c>
       <c r="D31" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,10),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E31" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,10),$T$5:$T$17,0))</f>
@@ -28202,11 +28238,11 @@
       </c>
       <c r="C32" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,11),$T$5:$T$17,0))</f>
-        <v>-0.276223776223776</v>
+        <v>-0.295454545454545</v>
       </c>
       <c r="D32" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,11),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E32" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,11),$T$5:$T$17,0))</f>
@@ -28228,11 +28264,11 @@
       </c>
       <c r="C33" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,12),$T$5:$T$17,0))</f>
-        <v>-0.307692307692308</v>
+        <v>-0.321428571428571</v>
       </c>
       <c r="D33" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,12),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E33" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,12),$T$5:$T$17,0))</f>
@@ -28254,11 +28290,11 @@
       </c>
       <c r="C34" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,13),$T$5:$T$17,0))</f>
-        <v>-0.346153846153846</v>
+        <v>-0.357142857142857</v>
       </c>
       <c r="D34" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,13),$T$5:$T$17,0))</f>
-        <v>0.8125</v>
+        <v>0.875</v>
       </c>
       <c r="E34" s="54" t="n">
         <f aca="false">INDEX($J$5:$J$17,MATCH(LARGE($T$5:$T$17,13),$T$5:$T$17,0))</f>
@@ -28368,7 +28404,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -28756,6 +28792,23 @@
       </c>
       <c r="E35" s="58" t="s">
         <v>209</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="58" t="s">
+        <v>160</v>
+      </c>
+      <c r="B36" s="58" t="s">
+        <v>210</v>
+      </c>
+      <c r="C36" s="58" t="s">
+        <v>211</v>
+      </c>
+      <c r="D36" s="58" t="s">
+        <v>212</v>
+      </c>
+      <c r="E36" s="58" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -28790,23 +28843,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="47" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B3" s="63" t="n">
         <v>0.1</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B4" s="64" t="n">
         <v>2</v>
@@ -28814,18 +28867,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="40" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B5" s="65" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28952,12 +29005,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28965,40 +29018,40 @@
         <v>59</v>
       </c>
       <c r="B4" s="66" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C4" s="66" t="s">
         <v>60</v>
       </c>
       <c r="D4" s="66" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="E4" s="66" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="F4" s="66" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="G4" s="66" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="H4" s="66" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="I4" s="66" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="J4" s="66" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="K4" s="66" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="L4" s="66" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="M4" s="66" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="N4" s="66" t="s">
         <v>46</v>
@@ -29068,79 +29121,79 @@
       <c r="L5" s="66"/>
       <c r="M5" s="66"/>
       <c r="N5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="O5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="P5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="Q5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="R5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="S5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="T5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="U5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="V5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="W5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="X5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="Y5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="Z5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="AA5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AB5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="AC5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AD5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="AE5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AF5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="AG5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AH5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="AI5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AJ5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="AK5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AL5" s="67" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="AM5" s="67" t="s">
         <v>102</v>
@@ -29148,28 +29201,28 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="68" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B6" s="69" t="s">
         <v>74</v>
       </c>
       <c r="C6" s="69" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D6" s="68" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F6" s="69" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G6" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="I6" s="71" t="n">
         <v>1</v>
@@ -29288,22 +29341,22 @@
         <v>74</v>
       </c>
       <c r="C7" s="69" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="D7" s="68" t="s">
+        <v>242</v>
+      </c>
+      <c r="E7" s="70" t="s">
         <v>238</v>
       </c>
-      <c r="E7" s="70" t="s">
-        <v>234</v>
-      </c>
       <c r="F7" s="69" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="G7" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I7" s="71" t="n">
         <v>5602.9</v>
@@ -29418,22 +29471,22 @@
         <v>74</v>
       </c>
       <c r="C8" s="69" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D8" s="68" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F8" s="69" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="G8" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="I8" s="71" t="n">
         <v>3.79</v>
@@ -29548,20 +29601,20 @@
         <v>74</v>
       </c>
       <c r="C9" s="69" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D9" s="68" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F9" s="69" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="G9" s="70"/>
       <c r="H9" s="70" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="I9" s="71"/>
       <c r="J9" s="71"/>
@@ -29648,20 +29701,20 @@
         <v>74</v>
       </c>
       <c r="C10" s="69" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D10" s="68" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="G10" s="70"/>
       <c r="H10" s="70" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I10" s="71"/>
       <c r="J10" s="71"/>
@@ -29742,28 +29795,28 @@
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="75" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B11" s="76" t="s">
         <v>76</v>
       </c>
       <c r="C11" s="76" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="D11" s="75" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F11" s="76" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G11" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H11" s="70" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="I11" s="71" t="n">
         <v>1</v>
@@ -29882,22 +29935,22 @@
         <v>76</v>
       </c>
       <c r="C12" s="76" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="D12" s="75" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F12" s="76" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="G12" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="I12" s="71" t="n">
         <v>36.92</v>
@@ -30012,22 +30065,22 @@
         <v>76</v>
       </c>
       <c r="C13" s="76" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D13" s="75" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F13" s="76" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="G13" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I13" s="71" t="n">
         <v>2956.72</v>
@@ -30136,28 +30189,28 @@
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="77" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B14" s="78" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C14" s="78" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="D14" s="77" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F14" s="78" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G14" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="I14" s="71" t="n">
         <v>1</v>
@@ -30273,25 +30326,25 @@
         <v>194</v>
       </c>
       <c r="B15" s="78" t="s">
+        <v>261</v>
+      </c>
+      <c r="C15" s="78" t="s">
+        <v>263</v>
+      </c>
+      <c r="D15" s="77" t="s">
+        <v>246</v>
+      </c>
+      <c r="E15" s="70" t="s">
+        <v>238</v>
+      </c>
+      <c r="F15" s="78" t="s">
         <v>257</v>
-      </c>
-      <c r="C15" s="78" t="s">
-        <v>259</v>
-      </c>
-      <c r="D15" s="77" t="s">
-        <v>242</v>
-      </c>
-      <c r="E15" s="70" t="s">
-        <v>234</v>
-      </c>
-      <c r="F15" s="78" t="s">
-        <v>253</v>
       </c>
       <c r="G15" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="I15" s="71" t="n">
         <v>38.11</v>
@@ -30403,25 +30456,25 @@
         <v>158</v>
       </c>
       <c r="B16" s="78" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C16" s="78" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D16" s="77" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="E16" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F16" s="78" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="G16" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I16" s="71" t="n">
         <v>33.22</v>
@@ -30533,25 +30586,25 @@
         <v>142</v>
       </c>
       <c r="B17" s="80" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C17" s="80" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="D17" s="79" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F17" s="80" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G17" s="70" t="n">
         <v>2023</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I17" s="71" t="n">
         <v>74620.05</v>
@@ -30663,25 +30716,25 @@
         <v>138</v>
       </c>
       <c r="B18" s="80" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C18" s="80" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D18" s="79" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E18" s="70" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="F18" s="80" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G18" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="I18" s="71" t="n">
         <v>11.89</v>
@@ -30793,25 +30846,25 @@
         <v>199</v>
       </c>
       <c r="B19" s="80" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C19" s="80" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="D19" s="79" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="E19" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F19" s="80" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="G19" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I19" s="71" t="n">
         <v>31.51</v>
@@ -30923,25 +30976,25 @@
         <v>202</v>
       </c>
       <c r="B20" s="80" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C20" s="80" t="s">
+        <v>274</v>
+      </c>
+      <c r="D20" s="79" t="s">
+        <v>252</v>
+      </c>
+      <c r="E20" s="70" t="s">
         <v>270</v>
       </c>
-      <c r="D20" s="79" t="s">
-        <v>248</v>
-      </c>
-      <c r="E20" s="70" t="s">
-        <v>266</v>
-      </c>
       <c r="F20" s="80" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="G20" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I20" s="83" t="n">
         <v>0.1254</v>
@@ -31053,104 +31106,134 @@
         <v>160</v>
       </c>
       <c r="B21" s="80" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C21" s="80" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="D21" s="79" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E21" s="70" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F21" s="80" t="s">
-        <v>272</v>
-      </c>
-      <c r="G21" s="70"/>
+        <v>276</v>
+      </c>
+      <c r="G21" s="70" t="n">
+        <v>2022</v>
+      </c>
       <c r="H21" s="70" t="s">
-        <v>244</v>
-      </c>
-      <c r="I21" s="71"/>
+        <v>248</v>
+      </c>
+      <c r="I21" s="71" t="n">
+        <v>18.24</v>
+      </c>
       <c r="J21" s="71"/>
       <c r="K21" s="71"/>
-      <c r="L21" s="72" t="str">
+      <c r="L21" s="72" t="n">
         <f aca="false">IF($H21="Absoluto",IF($J21="","",$J21),IF($I21="","",IF($H21="Razão MT",MIN($I21*(1-Parâmetros!$B$3),$I21*(1+Parâmetros!$B$3)),$I21-Parâmetros!$B$4)))</f>
-        <v/>
-      </c>
-      <c r="M21" s="72" t="str">
+        <v>16.24</v>
+      </c>
+      <c r="M21" s="72" t="n">
         <f aca="false">IF($H21="Absoluto",IF($K21="","",$K21),IF($I21="","",IF($H21="Razão MT",MAX($I21*(1-Parâmetros!$B$3),$I21*(1+Parâmetros!$B$3)),$I21+Parâmetros!$B$4)))</f>
-        <v/>
-      </c>
-      <c r="N21" s="71"/>
+        <v>20.24</v>
+      </c>
+      <c r="N21" s="71" t="n">
+        <v>6.34</v>
+      </c>
       <c r="O21" s="74" t="str">
         <f aca="false">IF(OR(N21="",$L21="",$M21=""),"",IF($E21="+",IF(N21&gt;$M21,"Força",IF(N21&lt;$L21,"Fraqueza","Neutro")),IF(N21&lt;$L21,"Força",IF(N21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="P21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="P21" s="71" t="n">
+        <v>17.68</v>
+      </c>
       <c r="Q21" s="74" t="str">
         <f aca="false">IF(OR(P21="",$L21="",$M21=""),"",IF($E21="+",IF(P21&gt;$M21,"Força",IF(P21&lt;$L21,"Fraqueza","Neutro")),IF(P21&lt;$L21,"Força",IF(P21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="R21" s="71"/>
+        <v>Neutro</v>
+      </c>
+      <c r="R21" s="71" t="n">
+        <v>5.5</v>
+      </c>
       <c r="S21" s="74" t="str">
         <f aca="false">IF(OR(R21="",$L21="",$M21=""),"",IF($E21="+",IF(R21&gt;$M21,"Força",IF(R21&lt;$L21,"Fraqueza","Neutro")),IF(R21&lt;$L21,"Força",IF(R21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="T21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="T21" s="71" t="n">
+        <v>5.76</v>
+      </c>
       <c r="U21" s="74" t="str">
         <f aca="false">IF(OR(T21="",$L21="",$M21=""),"",IF($E21="+",IF(T21&gt;$M21,"Força",IF(T21&lt;$L21,"Fraqueza","Neutro")),IF(T21&lt;$L21,"Força",IF(T21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="V21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="V21" s="71" t="n">
+        <v>11.87</v>
+      </c>
       <c r="W21" s="74" t="str">
         <f aca="false">IF(OR(V21="",$L21="",$M21=""),"",IF($E21="+",IF(V21&gt;$M21,"Força",IF(V21&lt;$L21,"Fraqueza","Neutro")),IF(V21&lt;$L21,"Força",IF(V21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="X21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="X21" s="71" t="n">
+        <v>11.71</v>
+      </c>
       <c r="Y21" s="74" t="str">
         <f aca="false">IF(OR(X21="",$L21="",$M21=""),"",IF($E21="+",IF(X21&gt;$M21,"Força",IF(X21&lt;$L21,"Fraqueza","Neutro")),IF(X21&lt;$L21,"Força",IF(X21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="Z21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="Z21" s="71" t="n">
+        <v>7.14</v>
+      </c>
       <c r="AA21" s="74" t="str">
         <f aca="false">IF(OR(Z21="",$L21="",$M21=""),"",IF($E21="+",IF(Z21&gt;$M21,"Força",IF(Z21&lt;$L21,"Fraqueza","Neutro")),IF(Z21&lt;$L21,"Força",IF(Z21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="AB21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="AB21" s="71" t="n">
+        <v>14.35</v>
+      </c>
       <c r="AC21" s="74" t="str">
         <f aca="false">IF(OR(AB21="",$L21="",$M21=""),"",IF($E21="+",IF(AB21&gt;$M21,"Força",IF(AB21&lt;$L21,"Fraqueza","Neutro")),IF(AB21&lt;$L21,"Força",IF(AB21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="AD21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="AD21" s="71" t="n">
+        <v>5.15</v>
+      </c>
       <c r="AE21" s="74" t="str">
         <f aca="false">IF(OR(AD21="",$L21="",$M21=""),"",IF($E21="+",IF(AD21&gt;$M21,"Força",IF(AD21&lt;$L21,"Fraqueza","Neutro")),IF(AD21&lt;$L21,"Força",IF(AD21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="AF21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="AF21" s="71" t="n">
+        <v>9.51</v>
+      </c>
       <c r="AG21" s="74" t="str">
         <f aca="false">IF(OR(AF21="",$L21="",$M21=""),"",IF($E21="+",IF(AF21&gt;$M21,"Força",IF(AF21&lt;$L21,"Fraqueza","Neutro")),IF(AF21&lt;$L21,"Força",IF(AF21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="AH21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="AH21" s="71" t="n">
+        <v>6.54</v>
+      </c>
       <c r="AI21" s="74" t="str">
         <f aca="false">IF(OR(AH21="",$L21="",$M21=""),"",IF($E21="+",IF(AH21&gt;$M21,"Força",IF(AH21&lt;$L21,"Fraqueza","Neutro")),IF(AH21&lt;$L21,"Força",IF(AH21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="AJ21" s="71"/>
+        <v>Fraqueza</v>
+      </c>
+      <c r="AJ21" s="71" t="n">
+        <v>21.61</v>
+      </c>
       <c r="AK21" s="74" t="str">
         <f aca="false">IF(OR(AJ21="",$L21="",$M21=""),"",IF($E21="+",IF(AJ21&gt;$M21,"Força",IF(AJ21&lt;$L21,"Fraqueza","Neutro")),IF(AJ21&lt;$L21,"Força",IF(AJ21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
-      </c>
-      <c r="AL21" s="71"/>
+        <v>Força</v>
+      </c>
+      <c r="AL21" s="71" t="n">
+        <v>9.96</v>
+      </c>
       <c r="AM21" s="74" t="str">
         <f aca="false">IF(OR(AL21="",$L21="",$M21=""),"",IF($E21="+",IF(AL21&gt;$M21,"Força",IF(AL21&lt;$L21,"Fraqueza","Neutro")),IF(AL21&lt;$L21,"Força",IF(AL21&gt;$M21,"Fraqueza","Neutro"))))</f>
-        <v/>
+        <v>Fraqueza</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="33" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -31232,12 +31315,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31248,13 +31331,13 @@
         <v>67</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D4" s="84" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="84" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="F4" s="84" t="s">
         <v>46</v>
@@ -31298,24 +31381,24 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C6" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="F6" s="70" t="n">
         <v>1</v>
@@ -31359,19 +31442,19 @@
     </row>
     <row r="7" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C7" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="F7" s="70" t="n">
         <v>3</v>
@@ -31415,19 +31498,19 @@
     </row>
     <row r="8" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F8" s="70" t="n">
         <v>3</v>
@@ -31471,19 +31554,19 @@
     </row>
     <row r="9" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C9" s="28" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="F9" s="70" t="n">
         <v>0</v>
@@ -31527,19 +31610,19 @@
     </row>
     <row r="10" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="F10" s="70" t="n">
         <v>1</v>
@@ -31583,19 +31666,19 @@
     </row>
     <row r="11" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="F11" s="70" t="n">
         <v>2</v>
@@ -31639,19 +31722,19 @@
     </row>
     <row r="12" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="85" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B12" s="85" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C12" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D12" s="86" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="E12" s="86" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="F12" s="70" t="n">
         <v>3</v>
@@ -31695,19 +31778,19 @@
     </row>
     <row r="13" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="85" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B13" s="85" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C13" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D13" s="86" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="E13" s="86" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F13" s="70" t="n">
         <v>2</v>
@@ -31751,19 +31834,19 @@
     </row>
     <row r="14" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="85" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="B14" s="85" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C14" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D14" s="86" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="E14" s="86" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="F14" s="70" t="n">
         <v>2</v>
@@ -31807,19 +31890,19 @@
     </row>
     <row r="15" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="85" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B15" s="85" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C15" s="86" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D15" s="86" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="E15" s="86" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="F15" s="70" t="n">
         <v>1</v>
@@ -31863,19 +31946,19 @@
     </row>
     <row r="16" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="85" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="B16" s="85" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C16" s="86" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="D16" s="86" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="E16" s="86" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="F16" s="70" t="n">
         <v>3</v>
@@ -31919,7 +32002,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revisa AM-03 com dados de desmatamento e CAR e adiciona contexto ambiental
- AM-03: Barão de Melgaço 2->3, Poconé 2->3 e N. Sra. do Livramento 1->2,
  com base no desmatamento 2019-2023 (d4_desmatamento.csv) e na
  conformidade do CAR (d4_car.csv); evidência e revisão registradas.
- Página: bloco ambiental (desmatamento anual por bioma, CAR) e
  mortalidade infantil no contexto social.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLDtP5x9bnGnFC43EPUEKq
</commit_message>
<xml_diff>
--- a/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
+++ b/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
@@ -318,8 +318,54 @@
 </comments>
 </file>
 
+<file path=xl/comments9.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="F14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Nota revista de 2 para 3 em 25/09/2026: 188 km² desmatados em 2019–2023 (d4_desmatamento.csv); 1.0% dos imóveis do CAR em conformidade (d4_car.csv).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Nota revista de 1 para 2 em 25/09/2026: 117 km² desmatados em 2019–2023 (d4_desmatamento.csv); 0.6% dos imóveis do CAR em conformidade (d4_car.csv).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Nota revista de 2 para 3 em 25/09/2026: 185 km² desmatados em 2019–2023 (d4_desmatamento.csv); 1.2% dos imóveis do CAR em conformidade (d4_car.csv).</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="347">
   <si>
     <t xml:space="preserve">MATRIZ SWOT DO PERFIL ECONÔMICO-PRODUTIVO SETORIAL MUNICIPAL (PESM) — PANTANAL NORTE</t>
   </si>
@@ -963,6 +1009,21 @@
     <t xml:space="preserve">O cálculo com receita_propria_real ÷ receita_total_real reproduz a coluna (diferença &lt; 0,01 p.p.). Denominador diferente do previsto (receita total em vez de corrente): tratar como aproximação.</t>
   </si>
   <si>
+    <t xml:space="preserve">AM-03 (revisão)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2019–2023 / 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d4_desmatamento.csv (PRODES/MapBiomas) e d4_car.csv (SICAR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notas revistas com dados: Barão de Melgaço 2→3, Poconé 2→3, N. Sra. do Livramento 1→2. Os demais mantidos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barão (188 km²), Poconé (185 km²), Cáceres (181), Sto. Antônio do Leverger (170) e Livramento (117) concentram o desmatamento recente da região; a conformidade do CAR é baixa em todos (0,6%–3,7%).</t>
+  </si>
+  <si>
     <t xml:space="preserve">PARÂMETROS</t>
   </si>
   <si>
@@ -1251,7 +1312,7 @@
     <t xml:space="preserve">Exigências ambientais de mercados importadores e barreiras ligadas a desmatamento (ex.: EUDR)</t>
   </si>
   <si>
-    <t xml:space="preserve">Pesquisa web-based; Comex Stat. Evidências: Regulamento UE 2023/1115 (EUDR) exige rastreabilidade livre de desmatamento para carne e soja; maior exposição em municípios exportadores de grãos/carne (Itiquira, Rondonópolis, Cáceres, Sto. Antônio do Leverger).</t>
+    <t xml:space="preserve">Pesquisa web-based; Comex Stat. Evidências: Regulamento UE 2023/1115 (EUDR) exige rastreabilidade livre de desmatamento para carne e soja; maior exposição em municípios exportadores de grãos/carne (Itiquira, Rondonópolis, Cáceres, Sto. Antônio do Leverger). | Dados (d4_desmatamento.csv, d4_car.csv): desmatamento 2019–2023 — Barão de Melgaço 188 km²; Poconé 185 km²; Cáceres 181 km²; Santo Antônio do Leverger 170 km²; Nossa Senhora do Livramento 117 km²; Itiquira 56 km²; Porto Esperidião 35 km²; demais abaixo de 10 km². Só 0,6% a 3,7% dos imóveis do CAR estão em conformidade nos 13 municípios (2024).</t>
   </si>
   <si>
     <t xml:space="preserve">AM-04</t>
@@ -2554,7 +2615,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="B2" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Indicadores (F-W)'!$A$4:$AM$4,0),"")</f>
@@ -2563,7 +2624,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B3" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Fatores Externos (O-A)'!$A$4:$R$4,0),"")</f>
@@ -2575,7 +2636,7 @@
         <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>102</v>
@@ -2584,16 +2645,16 @@
         <v>31</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>59</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>67</v>
@@ -2602,16 +2663,16 @@
         <v>33</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3415,12 +3476,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4079,7 +4140,7 @@
       </c>
       <c r="S14" s="1" t="n">
         <f aca="false">IF('Fatores Externos (O-A)'!F14="","",'Fatores Externos (O-A)'!F14)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" s="1" t="n">
         <f aca="false">IF(AND(R14="Oportunidade",ISNUMBER(S14)),IF(S14&gt;=Parâmetros!$B$5,1,0),0)</f>
@@ -4555,7 +4616,7 @@
       </c>
       <c r="H26" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(3,$W$6:$W$16,0)),"")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4813,7 +4874,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -4859,12 +4920,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6257,7 +6318,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -6303,12 +6364,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7701,7 +7762,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -7747,12 +7808,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9145,7 +9206,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -9191,12 +9252,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10589,7 +10650,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -10635,12 +10696,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12033,7 +12094,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -12079,12 +12140,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13477,7 +13538,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -13523,12 +13584,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14921,7 +14982,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -14967,12 +15028,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15631,7 +15692,7 @@
       </c>
       <c r="S14" s="1" t="n">
         <f aca="false">IF('Fatores Externos (O-A)'!N14="","",'Fatores Externos (O-A)'!N14)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T14" s="1" t="n">
         <f aca="false">IF(AND(R14="Oportunidade",ISNUMBER(S14)),IF(S14&gt;=Parâmetros!$B$5,1,0),0)</f>
@@ -15643,11 +15704,11 @@
       </c>
       <c r="V14" s="1" t="n">
         <f aca="false">IF(AND(R14="Ameaça",ISNUMBER(S14)),IF(S14&gt;=Parâmetros!$B$5,1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="W14" s="1" t="str">
+        <v>1</v>
+      </c>
+      <c r="W14" s="1" t="n">
         <f aca="false">IF(V14=1,SUM(V$6:V14),"")</f>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15797,7 +15858,7 @@
       </c>
       <c r="W16" s="1" t="n">
         <f aca="false">IF(V16=1,SUM(V$6:V16),"")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16002,7 +16063,7 @@
       <c r="D22" s="23"/>
       <c r="F22" s="24" t="str">
         <f aca="false">"AMEAÇAS (T) — "&amp;SUM($V$6:$V$16)&amp;" item(ns)"</f>
-        <v>AMEAÇAS (T) — 3 item(ns)</v>
+        <v>AMEAÇAS (T) — 4 item(ns)</v>
       </c>
       <c r="G22" s="24"/>
       <c r="H22" s="24"/>
@@ -16103,11 +16164,11 @@
       </c>
       <c r="G26" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(3,$W$6:$W$16,0)),"")</f>
-        <v>[Comércio e Serviços] AM-05 – Polarização regional por centros maiores (evasão de consumo, serviços e mão de obra)</v>
+        <v>[Agropecuária] AM-03 – Exigências ambientais de mercados importadores e barreiras ligadas a desmatamento (ex.: EUDR)</v>
       </c>
       <c r="H26" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(3,$W$6:$W$16,0)),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16124,17 +16185,17 @@
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(4,$U$6:$U$16,0)),"")</f>
         <v>2</v>
       </c>
-      <c r="F27" s="30" t="str">
+      <c r="F27" s="30" t="n">
         <f aca="false">IF(G27="","",4)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G27" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(4,$W$6:$W$16,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H27" s="32" t="str">
+        <v>[Comércio e Serviços] AM-05 – Polarização regional por centros maiores (evasão de consumo, serviços e mão de obra)</v>
+      </c>
+      <c r="H27" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(4,$W$6:$W$16,0)),"")</f>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16365,7 +16426,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -17232,12 +17293,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17896,7 +17957,7 @@
       </c>
       <c r="S14" s="1" t="n">
         <f aca="false">IF('Fatores Externos (O-A)'!O14="","",'Fatores Externos (O-A)'!O14)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" s="1" t="n">
         <f aca="false">IF(AND(R14="Oportunidade",ISNUMBER(S14)),IF(S14&gt;=Parâmetros!$B$5,1,0),0)</f>
@@ -18372,7 +18433,7 @@
       </c>
       <c r="H26" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(3,$W$6:$W$16,0)),"")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18630,7 +18691,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -18676,12 +18737,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20074,7 +20135,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -20120,12 +20181,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21518,7 +21579,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -21564,12 +21625,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22962,7 +23023,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -23364,11 +23425,11 @@
       </c>
       <c r="H12" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Ameaça",'Fatores Externos (O-A)'!N$6:N$16,"&gt;="&amp;Parâmetros!$B$5)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I12" s="36" t="n">
         <f aca="false">G12-H12</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24240,11 +24301,11 @@
       </c>
       <c r="D48" s="36" t="n">
         <f aca="false">COUNTIF('Fatores Externos (O-A)'!$F14:$R14,"&gt;="&amp;Parâmetros!$B$5)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E48" s="39" t="n">
         <f aca="false">IF(COUNT('Fatores Externos (O-A)'!$F14:$R14)=0,"",AVERAGE('Fatores Externos (O-A)'!$F14:$R14))</f>
-        <v>2.15384615384615</v>
+        <v>2.38461538461538</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27667,7 +27728,7 @@
       </c>
       <c r="H13" s="53" t="n">
         <f aca="false">Painel!H12</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I13" s="53" t="n">
         <f aca="false">COUNT('Fatores Externos (O-A)'!N$6:N$16)</f>
@@ -27679,15 +27740,15 @@
       </c>
       <c r="K13" s="55" t="n">
         <f aca="false">IF(I13=0,"",(G13-H13)/I13)</f>
-        <v>0.0909090909090909</v>
+        <v>0</v>
       </c>
       <c r="L13" s="56" t="n">
         <f aca="false">IF(F13="","",IF(K13="",F13,(F13+K13)/2))</f>
-        <v>-0.0974025974025974</v>
+        <v>-0.142857142857143</v>
       </c>
       <c r="M13" s="46" t="n">
         <f aca="false">IF(L13="","",RANK(L13,$L$5:$L$17,0))</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N13" s="49" t="str">
         <f aca="false">IF(AND(E13&gt;=0.75,J13&gt;=0.75),"Consolidado","PROVISÓRIO")</f>
@@ -27695,7 +27756,7 @@
       </c>
       <c r="T13" s="1" t="n">
         <f aca="false">IF(L13="",-9,L13)-ROW()*0.000000001</f>
-        <v>-0.0974026104025974</v>
+        <v>-0.142857155857143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28100,7 +28161,7 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="46" t="n">
         <f aca="false">INDEX($M$5:$M$17,MATCH(LARGE($T$5:$T$17,6),$T$5:$T$17,0))</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B27" s="38" t="str">
         <f aca="false">INDEX($A$5:$A$17,MATCH(LARGE($T$5:$T$17,6),$T$5:$T$17,0))</f>
@@ -28108,7 +28169,7 @@
       </c>
       <c r="C27" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,6),$T$5:$T$17,0))</f>
-        <v>-0.0974025974025974</v>
+        <v>-0.142857142857143</v>
       </c>
       <c r="D27" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,6),$T$5:$T$17,0))</f>
@@ -28404,7 +28465,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -28809,6 +28870,23 @@
       </c>
       <c r="E36" s="58" t="s">
         <v>213</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="58" t="s">
+        <v>214</v>
+      </c>
+      <c r="B37" s="58" t="s">
+        <v>215</v>
+      </c>
+      <c r="C37" s="58" t="s">
+        <v>216</v>
+      </c>
+      <c r="D37" s="58" t="s">
+        <v>217</v>
+      </c>
+      <c r="E37" s="58" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -28843,23 +28921,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="47" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B3" s="63" t="n">
         <v>0.1</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B4" s="64" t="n">
         <v>2</v>
@@ -28867,18 +28945,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="40" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B5" s="65" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29005,12 +29083,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29018,40 +29096,40 @@
         <v>59</v>
       </c>
       <c r="B4" s="66" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="C4" s="66" t="s">
         <v>60</v>
       </c>
       <c r="D4" s="66" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="E4" s="66" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="F4" s="66" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="G4" s="66" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="H4" s="66" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="I4" s="66" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="J4" s="66" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="K4" s="66" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="L4" s="66" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="M4" s="66" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="N4" s="66" t="s">
         <v>46</v>
@@ -29121,79 +29199,79 @@
       <c r="L5" s="66"/>
       <c r="M5" s="66"/>
       <c r="N5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="O5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="P5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="Q5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="R5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="S5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="T5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="U5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="V5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="W5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="X5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="Y5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="Z5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="AA5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AB5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="AC5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AD5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="AE5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AF5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="AG5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AH5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="AI5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AJ5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="AK5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AL5" s="67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="AM5" s="67" t="s">
         <v>102</v>
@@ -29201,28 +29279,28 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="68" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B6" s="69" t="s">
         <v>74</v>
       </c>
       <c r="C6" s="69" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="D6" s="68" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F6" s="69" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="G6" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="I6" s="71" t="n">
         <v>1</v>
@@ -29341,22 +29419,22 @@
         <v>74</v>
       </c>
       <c r="C7" s="69" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D7" s="68" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F7" s="69" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="G7" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I7" s="71" t="n">
         <v>5602.9</v>
@@ -29471,22 +29549,22 @@
         <v>74</v>
       </c>
       <c r="C8" s="69" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="D8" s="68" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F8" s="69" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="G8" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="I8" s="71" t="n">
         <v>3.79</v>
@@ -29601,20 +29679,20 @@
         <v>74</v>
       </c>
       <c r="C9" s="69" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D9" s="68" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F9" s="69" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="G9" s="70"/>
       <c r="H9" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="I9" s="71"/>
       <c r="J9" s="71"/>
@@ -29701,20 +29779,20 @@
         <v>74</v>
       </c>
       <c r="C10" s="69" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D10" s="68" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="G10" s="70"/>
       <c r="H10" s="70" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I10" s="71"/>
       <c r="J10" s="71"/>
@@ -29795,28 +29873,28 @@
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="75" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B11" s="76" t="s">
         <v>76</v>
       </c>
       <c r="C11" s="76" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D11" s="75" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F11" s="76" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="G11" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H11" s="70" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="I11" s="71" t="n">
         <v>1</v>
@@ -29935,22 +30013,22 @@
         <v>76</v>
       </c>
       <c r="C12" s="76" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D12" s="75" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F12" s="76" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="G12" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="I12" s="71" t="n">
         <v>36.92</v>
@@ -30065,22 +30143,22 @@
         <v>76</v>
       </c>
       <c r="C13" s="76" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D13" s="75" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F13" s="76" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="G13" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I13" s="71" t="n">
         <v>2956.72</v>
@@ -30189,28 +30267,28 @@
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="77" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B14" s="78" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="C14" s="78" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="D14" s="77" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F14" s="78" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="G14" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="I14" s="71" t="n">
         <v>1</v>
@@ -30326,25 +30404,25 @@
         <v>194</v>
       </c>
       <c r="B15" s="78" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="C15" s="78" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D15" s="77" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F15" s="78" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="G15" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="I15" s="71" t="n">
         <v>38.11</v>
@@ -30456,25 +30534,25 @@
         <v>158</v>
       </c>
       <c r="B16" s="78" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="C16" s="78" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="D16" s="77" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="E16" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F16" s="78" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G16" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I16" s="71" t="n">
         <v>33.22</v>
@@ -30586,25 +30664,25 @@
         <v>142</v>
       </c>
       <c r="B17" s="80" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C17" s="80" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="D17" s="79" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F17" s="80" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="G17" s="70" t="n">
         <v>2023</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I17" s="71" t="n">
         <v>74620.05</v>
@@ -30716,25 +30794,25 @@
         <v>138</v>
       </c>
       <c r="B18" s="80" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C18" s="80" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="D18" s="79" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="E18" s="70" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="F18" s="80" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="G18" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="I18" s="71" t="n">
         <v>11.89</v>
@@ -30846,25 +30924,25 @@
         <v>199</v>
       </c>
       <c r="B19" s="80" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C19" s="80" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D19" s="79" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="E19" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F19" s="80" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="G19" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I19" s="71" t="n">
         <v>31.51</v>
@@ -30976,25 +31054,25 @@
         <v>202</v>
       </c>
       <c r="B20" s="80" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C20" s="80" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="D20" s="79" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E20" s="70" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="F20" s="80" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="G20" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I20" s="83" t="n">
         <v>0.1254</v>
@@ -31106,25 +31184,25 @@
         <v>160</v>
       </c>
       <c r="B21" s="80" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C21" s="80" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D21" s="79" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="E21" s="70" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F21" s="80" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G21" s="70" t="n">
         <v>2022</v>
       </c>
       <c r="H21" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="I21" s="71" t="n">
         <v>18.24</v>
@@ -31233,7 +31311,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="33" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -31315,12 +31393,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31331,13 +31409,13 @@
         <v>67</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="D4" s="84" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="84" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="F4" s="84" t="s">
         <v>46</v>
@@ -31381,24 +31459,24 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C6" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="F6" s="70" t="n">
         <v>1</v>
@@ -31442,19 +31520,19 @@
     </row>
     <row r="7" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C7" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="F7" s="70" t="n">
         <v>3</v>
@@ -31498,19 +31576,19 @@
     </row>
     <row r="8" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="F8" s="70" t="n">
         <v>3</v>
@@ -31554,19 +31632,19 @@
     </row>
     <row r="9" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C9" s="28" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="F9" s="70" t="n">
         <v>0</v>
@@ -31610,19 +31688,19 @@
     </row>
     <row r="10" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="F10" s="70" t="n">
         <v>1</v>
@@ -31666,19 +31744,19 @@
     </row>
     <row r="11" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="F11" s="70" t="n">
         <v>2</v>
@@ -31722,19 +31800,19 @@
     </row>
     <row r="12" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="85" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="B12" s="85" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C12" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D12" s="86" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="E12" s="86" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="F12" s="70" t="n">
         <v>3</v>
@@ -31778,19 +31856,19 @@
     </row>
     <row r="13" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="85" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B13" s="85" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C13" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D13" s="86" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="E13" s="86" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="F13" s="70" t="n">
         <v>2</v>
@@ -31834,22 +31912,22 @@
     </row>
     <row r="14" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="85" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B14" s="85" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C14" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D14" s="86" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="E14" s="86" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="F14" s="70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" s="70" t="n">
         <v>3</v>
@@ -31873,10 +31951,10 @@
         <v>1</v>
       </c>
       <c r="N14" s="70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" s="70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" s="70" t="n">
         <v>2</v>
@@ -31890,19 +31968,19 @@
     </row>
     <row r="15" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="85" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B15" s="85" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C15" s="86" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D15" s="86" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="E15" s="86" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="F15" s="70" t="n">
         <v>1</v>
@@ -31946,19 +32024,19 @@
     </row>
     <row r="16" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="85" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="B16" s="85" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C16" s="86" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D16" s="86" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="E16" s="86" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="F16" s="70" t="n">
         <v>3</v>
@@ -32002,7 +32080,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -32024,5 +32102,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revisa AM-01, OP-01 e OP-05 com queimadas, comércio exterior e rodovias
- AM-01: Itiquira e Porto Esperidião 2->1 (focos 2013-2022 abaixo da
  média de MT); série de 2023-2024 descartada por quebra de escala.
- OP-01: Mirassol D'Oeste 2->3 (carne bovina congelada é o principal
  produto exportado). OP-05: Sto. Antônio do Leverger 2->3 (BR-163/364
  duplicada).
- Página: focos de calor por ano, quadros de infraestrutura (rodovias e
  energia) e produto principal no tooltip das exportações.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLDtP5x9bnGnFC43EPUEKq
</commit_message>
<xml_diff>
--- a/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
+++ b/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
@@ -336,6 +336,30 @@
         </r>
       </text>
     </comment>
+    <comment ref="J12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Nota revista de 2 para 1 em 25/09/2026. Focos de calor 2013–2022: 11,5 por mil km²/ano, abaixo da média de MT (30,9) (d4_queimadas.csv).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M6" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Nota revista de 2 para 3 em 25/09/2026. Carne bovina congelada (SH4 0202) é o principal produto exportado: 65%–78% de US$ 108–184 milhões/ano em 2022–2024 (d2_comercio_exterior.csv).</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="N14" authorId="0">
       <text>
         <r>
@@ -360,12 +384,36 @@
         </r>
       </text>
     </comment>
+    <comment ref="P12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Nota revista de 2 para 1 em 25/09/2026. Focos de calor 2013–2022: 16,1 por mil km²/ano, abaixo da média de MT (30,9) (d4_queimadas.csv).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Nota revista de 2 para 3 em 25/09/2026. 133 km de rodovia duplicada (BR-163/364) e 98% da malha pavimentada (d5_rodovias.csv).</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="352">
   <si>
     <t xml:space="preserve">MATRIZ SWOT DO PERFIL ECONÔMICO-PRODUTIVO SETORIAL MUNICIPAL (PESM) — PANTANAL NORTE</t>
   </si>
@@ -1024,6 +1072,21 @@
     <t xml:space="preserve">Barão (188 km²), Poconé (185 km²), Cáceres (181), Sto. Antônio do Leverger (170) e Livramento (117) concentram o desmatamento recente da região; a conformidade do CAR é baixa em todos (0,6%–3,7%).</t>
   </si>
   <si>
+    <t xml:space="preserve">AM-01, OP-01, OP-05 (revisão)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2013–2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d4_queimadas.csv, d2_comercio_exterior.csv, d5_rodovias.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notas revistas com dados: AM-01 Itiquira 2→1; AM-01 Porto Esperidião 2→1; OP-01 Mirassol D'Oeste 2→3; OP-05 Santo Antônio do Leverger 2→3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Série de focos de 2023–2024 com quebra de escala (total de MT passa de ~30 mil para 0,7–1,7 milhão/ano): usar só para comparar municípios dentro do mesmo ano. d5_energia.csv mostra consumo industrial alto em Poconé (46%) e N. Sra. do Livramento (43%), ligado à mineração de ouro, não à agroindústria.</t>
+  </si>
+  <si>
     <t xml:space="preserve">PARÂMETROS</t>
   </si>
   <si>
@@ -1237,7 +1300,7 @@
     <t xml:space="preserve">Demanda externa por carne bovina e proteína animal</t>
   </si>
   <si>
-    <t xml:space="preserve">Comex Stat; IMEA; Cepea. Evidências: MT tem o maior rebanho do país (≈34 mi cab., 14,2% do BR – IBGE/PPM 2023); Cáceres é o maior rebanho de MT (≈1,4 mi cab., 4º do Brasil). Nota maior onde o QL agro e o rebanho são altos (Cáceres, Porto Esperidião, Sto. Antônio do Leverger).</t>
+    <t xml:space="preserve">Comex Stat; IMEA; Cepea. Evidências: MT tem o maior rebanho do país (≈34 mi cab., 14,2% do BR – IBGE/PPM 2023); Cáceres é o maior rebanho de MT (≈1,4 mi cab., 4º do Brasil). Nota maior onde o QL agro e o rebanho são altos (Cáceres, Porto Esperidião, Sto. Antônio do Leverger). | Dados (d2_comercio_exterior.csv): Mirassol D'Oeste exporta sobretudo carne bovina congelada (SH4 0202); Cáceres, madeira serrada (4407); Itiquira, soja (1201); Rondonópolis, farelo de soja (2304); Poconé e N. Sra. do Livramento, ouro (7108).</t>
   </si>
   <si>
     <t xml:space="preserve">OP-02</t>
@@ -1273,7 +1336,7 @@
     <t xml:space="preserve">Corredores logísticos (rodovias federais, ferrovia, hidrovia do Paraguai)</t>
   </si>
   <si>
-    <t xml:space="preserve">DNIT; ANTT; ANTAQ; pesquisa web-based. Evidências: Ferrovia Estadual Rondonópolis–Lucas do Rio Verde (Rumo; R$ 2 bi em 2025, trecho até Campo Verde previsto p/ 2026 – Rumo/BNDES); Porto de Cáceres reformado e terminal Paratudal em licenciamento (hidrovia Paraguai–Paraná); BR-163/364 (Rondonópolis, Itiquira, Juscimeira) e BR-070/174 (Cáceres, Livramento, Mirassol, Porto Esperidião).</t>
+    <t xml:space="preserve">DNIT; ANTT; ANTAQ; pesquisa web-based. Evidências: Ferrovia Estadual Rondonópolis–Lucas do Rio Verde (Rumo; R$ 2 bi em 2025, trecho até Campo Verde previsto p/ 2026 – Rumo/BNDES); Porto de Cáceres reformado e terminal Paratudal em licenciamento (hidrovia Paraguai–Paraná); BR-163/364 (Rondonópolis, Itiquira, Juscimeira) e BR-070/174 (Cáceres, Livramento, Mirassol, Porto Esperidião). | Dados (d5_rodovias.csv): rodovia duplicada em Rondonópolis (291 km), Itiquira (134), Sto. Antônio do Leverger (133) e Juscimeira (69); malha pavimentada abaixo de 40% em Lambari D'Oeste e Porto Esperidião.</t>
   </si>
   <si>
     <t xml:space="preserve">OP-06</t>
@@ -1294,7 +1357,7 @@
     <t xml:space="preserve">Eventos climáticos extremos: secas prolongadas e incêndios no Pantanal</t>
   </si>
   <si>
-    <t xml:space="preserve">INPE – BDQueimadas; MapBiomas; Cemaden. Evidências: incêndios de 2024 – Cáceres ≈87 mil ha, Poconé ≈61,5 mil ha, Barão de Melgaço ≈2,6 mil ha (Bombeiros-MT/INPE); 2020 foi o pior ano da série no Pantanal; ≈95% dos focos de 2024 começaram em propriedades privadas. Planície pantaneira = exposição alta.</t>
+    <t xml:space="preserve">INPE – BDQueimadas; MapBiomas; Cemaden. Evidências: incêndios de 2024 – Cáceres ≈87 mil ha, Poconé ≈61,5 mil ha, Barão de Melgaço ≈2,6 mil ha (Bombeiros-MT/INPE); 2020 foi o pior ano da série no Pantanal; ≈95% dos focos de 2024 começaram em propriedades privadas. Planície pantaneira = exposição alta. | Dados (d4_queimadas.csv, 2013–2022; a série de 2023–2024 muda de escala e não foi usada): focos por mil km²/ano — Barão de Melgaço 64,5; Poconé 51,4; Sto. Antônio do Leverger 34,1; N. Sra. do Livramento 30,7; Cáceres 25,4; MT 30,9; demais abaixo de 17.</t>
   </si>
   <si>
     <t xml:space="preserve">AM-02</t>
@@ -2615,7 +2678,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B2" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Indicadores (F-W)'!$A$4:$AM$4,0),"")</f>
@@ -2624,7 +2687,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B3" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Fatores Externos (O-A)'!$A$4:$R$4,0),"")</f>
@@ -2636,7 +2699,7 @@
         <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>102</v>
@@ -2645,16 +2708,16 @@
         <v>31</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>59</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>67</v>
@@ -2663,16 +2726,16 @@
         <v>33</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3476,12 +3539,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4874,7 +4937,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -4920,12 +4983,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6318,7 +6381,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -6364,12 +6427,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7762,7 +7825,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -7808,12 +7871,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9206,7 +9269,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -9252,12 +9315,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9766,7 +9829,7 @@
       </c>
       <c r="S12" s="1" t="n">
         <f aca="false">IF('Fatores Externos (O-A)'!J12="","",'Fatores Externos (O-A)'!J12)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T12" s="1" t="n">
         <f aca="false">IF(AND(R12="Oportunidade",ISNUMBER(S12)),IF(S12&gt;=Parâmetros!$B$5,1,0),0)</f>
@@ -9778,11 +9841,11 @@
       </c>
       <c r="V12" s="1" t="n">
         <f aca="false">IF(AND(R12="Ameaça",ISNUMBER(S12)),IF(S12&gt;=Parâmetros!$B$5,1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="W12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="1" t="str">
         <f aca="false">IF(V12=1,SUM(V$6:V12),"")</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9857,7 +9920,7 @@
       </c>
       <c r="W13" s="1" t="n">
         <f aca="false">IF(V13=1,SUM(V$6:V13),"")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9932,7 +9995,7 @@
       </c>
       <c r="W14" s="1" t="n">
         <f aca="false">IF(V14=1,SUM(V$6:V14),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10007,7 +10070,7 @@
       </c>
       <c r="W15" s="1" t="n">
         <f aca="false">IF(V15=1,SUM(V$6:V15),"")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10082,7 +10145,7 @@
       </c>
       <c r="W16" s="1" t="n">
         <f aca="false">IF(V16=1,SUM(V$6:V16),"")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10287,7 +10350,7 @@
       <c r="D22" s="23"/>
       <c r="F22" s="24" t="str">
         <f aca="false">"AMEAÇAS (T) — "&amp;SUM($V$6:$V$16)&amp;" item(ns)"</f>
-        <v>AMEAÇAS (T) — 5 item(ns)</v>
+        <v>AMEAÇAS (T) — 4 item(ns)</v>
       </c>
       <c r="G22" s="24"/>
       <c r="H22" s="24"/>
@@ -10334,11 +10397,11 @@
       </c>
       <c r="G24" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(1,$W$6:$W$16,0)),"")</f>
-        <v>[Agropecuária] AM-01 – Eventos climáticos extremos: secas prolongadas e incêndios no Pantanal</v>
+        <v>[Agropecuária] AM-02 – Volatilidade de preços de commodities (boi gordo, soja, milho)</v>
       </c>
       <c r="H24" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(1,$W$6:$W$16,0)),"")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10361,7 +10424,7 @@
       </c>
       <c r="G25" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(2,$W$6:$W$16,0)),"")</f>
-        <v>[Agropecuária] AM-02 – Volatilidade de preços de commodities (boi gordo, soja, milho)</v>
+        <v>[Agropecuária] AM-03 – Exigências ambientais de mercados importadores e barreiras ligadas a desmatamento (ex.: EUDR)</v>
       </c>
       <c r="H25" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(2,$W$6:$W$16,0)),"")</f>
@@ -10388,7 +10451,7 @@
       </c>
       <c r="G26" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(3,$W$6:$W$16,0)),"")</f>
-        <v>[Agropecuária] AM-03 – Exigências ambientais de mercados importadores e barreiras ligadas a desmatamento (ex.: EUDR)</v>
+        <v>[Estrutura Econômica e Fiscal] AM-04 – Transição da Reforma Tributária (IBS/CBS) e efeitos sobre a repartição de receitas municipais</v>
       </c>
       <c r="H26" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(3,$W$6:$W$16,0)),"")</f>
@@ -10415,11 +10478,11 @@
       </c>
       <c r="G27" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(4,$W$6:$W$16,0)),"")</f>
-        <v>[Estrutura Econômica e Fiscal] AM-04 – Transição da Reforma Tributária (IBS/CBS) e efeitos sobre a repartição de receitas municipais</v>
+        <v>[Comércio e Serviços] AM-05 – Polarização regional por centros maiores (evasão de consumo, serviços e mão de obra)</v>
       </c>
       <c r="H27" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(4,$W$6:$W$16,0)),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10436,17 +10499,17 @@
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(5,$U$6:$U$16,0)),"")</f>
         <v>3</v>
       </c>
-      <c r="F28" s="30" t="n">
+      <c r="F28" s="30" t="str">
         <f aca="false">IF(G28="","",5)</f>
-        <v>5</v>
+        <v/>
       </c>
       <c r="G28" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(5,$W$6:$W$16,0)),"")</f>
-        <v>[Comércio e Serviços] AM-05 – Polarização regional por centros maiores (evasão de consumo, serviços e mão de obra)</v>
-      </c>
-      <c r="H28" s="32" t="n">
+        <v/>
+      </c>
+      <c r="H28" s="32" t="str">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(5,$W$6:$W$16,0)),"")</f>
-        <v>2</v>
+        <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10650,7 +10713,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -10696,12 +10759,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12094,7 +12157,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -12140,12 +12203,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13538,7 +13601,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -13584,12 +13647,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13653,7 +13716,7 @@
       </c>
       <c r="S6" s="1" t="n">
         <f aca="false">IF('Fatores Externos (O-A)'!M6="","",'Fatores Externos (O-A)'!M6)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T6" s="1" t="n">
         <f aca="false">IF(AND(R6="Oportunidade",ISNUMBER(S6)),IF(S6&gt;=Parâmetros!$B$5,1,0),0)</f>
@@ -14658,7 +14721,7 @@
       </c>
       <c r="D24" s="29" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(1,$U$6:$U$16,0)),"")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24" s="30" t="n">
         <f aca="false">IF(G24="","",1)</f>
@@ -14982,7 +15045,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -15028,12 +15091,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16426,7 +16489,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -17293,12 +17356,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18691,7 +18754,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -18737,12 +18800,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19251,7 +19314,7 @@
       </c>
       <c r="S12" s="1" t="n">
         <f aca="false">IF('Fatores Externos (O-A)'!P12="","",'Fatores Externos (O-A)'!P12)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T12" s="1" t="n">
         <f aca="false">IF(AND(R12="Oportunidade",ISNUMBER(S12)),IF(S12&gt;=Parâmetros!$B$5,1,0),0)</f>
@@ -19263,11 +19326,11 @@
       </c>
       <c r="V12" s="1" t="n">
         <f aca="false">IF(AND(R12="Ameaça",ISNUMBER(S12)),IF(S12&gt;=Parâmetros!$B$5,1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="W12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="1" t="str">
         <f aca="false">IF(V12=1,SUM(V$6:V12),"")</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19342,7 +19405,7 @@
       </c>
       <c r="W13" s="1" t="n">
         <f aca="false">IF(V13=1,SUM(V$6:V13),"")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19417,7 +19480,7 @@
       </c>
       <c r="W14" s="1" t="n">
         <f aca="false">IF(V14=1,SUM(V$6:V14),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19567,7 +19630,7 @@
       </c>
       <c r="W16" s="1" t="n">
         <f aca="false">IF(V16=1,SUM(V$6:V16),"")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19772,7 +19835,7 @@
       <c r="D22" s="23"/>
       <c r="F22" s="24" t="str">
         <f aca="false">"AMEAÇAS (T) — "&amp;SUM($V$6:$V$16)&amp;" item(ns)"</f>
-        <v>AMEAÇAS (T) — 4 item(ns)</v>
+        <v>AMEAÇAS (T) — 3 item(ns)</v>
       </c>
       <c r="G22" s="24"/>
       <c r="H22" s="24"/>
@@ -19819,11 +19882,11 @@
       </c>
       <c r="G24" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(1,$W$6:$W$16,0)),"")</f>
-        <v>[Agropecuária] AM-01 – Eventos climáticos extremos: secas prolongadas e incêndios no Pantanal</v>
+        <v>[Agropecuária] AM-02 – Volatilidade de preços de commodities (boi gordo, soja, milho)</v>
       </c>
       <c r="H24" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(1,$W$6:$W$16,0)),"")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19846,11 +19909,11 @@
       </c>
       <c r="G25" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(2,$W$6:$W$16,0)),"")</f>
-        <v>[Agropecuária] AM-02 – Volatilidade de preços de commodities (boi gordo, soja, milho)</v>
+        <v>[Agropecuária] AM-03 – Exigências ambientais de mercados importadores e barreiras ligadas a desmatamento (ex.: EUDR)</v>
       </c>
       <c r="H25" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(2,$W$6:$W$16,0)),"")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19873,7 +19936,7 @@
       </c>
       <c r="G26" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(3,$W$6:$W$16,0)),"")</f>
-        <v>[Agropecuária] AM-03 – Exigências ambientais de mercados importadores e barreiras ligadas a desmatamento (ex.: EUDR)</v>
+        <v>[Comércio e Serviços] AM-05 – Polarização regional por centros maiores (evasão de consumo, serviços e mão de obra)</v>
       </c>
       <c r="H26" s="32" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(3,$W$6:$W$16,0)),"")</f>
@@ -19894,17 +19957,17 @@
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(4,$U$6:$U$16,0)),"")</f>
         <v/>
       </c>
-      <c r="F27" s="30" t="n">
+      <c r="F27" s="30" t="str">
         <f aca="false">IF(G27="","",4)</f>
-        <v>4</v>
+        <v/>
       </c>
       <c r="G27" s="31" t="str">
         <f aca="false">IFERROR(INDEX($Q$6:$Q$16,MATCH(4,$W$6:$W$16,0)),"")</f>
-        <v>[Comércio e Serviços] AM-05 – Polarização regional por centros maiores (evasão de consumo, serviços e mão de obra)</v>
-      </c>
-      <c r="H27" s="32" t="n">
+        <v/>
+      </c>
+      <c r="H27" s="32" t="str">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(4,$W$6:$W$16,0)),"")</f>
-        <v>2</v>
+        <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20135,7 +20198,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -20181,12 +20244,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21579,7 +21642,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -21625,12 +21688,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21989,7 +22052,7 @@
       </c>
       <c r="S10" s="1" t="n">
         <f aca="false">IF('Fatores Externos (O-A)'!R10="","",'Fatores Externos (O-A)'!R10)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="1" t="n">
         <f aca="false">IF(AND(R10="Oportunidade",ISNUMBER(S10)),IF(S10&gt;=Parâmetros!$B$5,1,0),0)</f>
@@ -22780,7 +22843,7 @@
       </c>
       <c r="D27" s="29" t="n">
         <f aca="false">IFERROR(INDEX($S$6:$S$16,MATCH(4,$U$6:$U$16,0)),"")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27" s="30" t="n">
         <f aca="false">IF(G27="","",4)</f>
@@ -23023,7 +23086,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -23277,11 +23340,11 @@
       </c>
       <c r="H8" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Ameaça",'Fatores Externos (O-A)'!J$6:J$16,"&gt;="&amp;Parâmetros!$B$5)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I8" s="36" t="n">
         <f aca="false">G8-H8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23499,11 +23562,11 @@
       </c>
       <c r="H14" s="36" t="n">
         <f aca="false">COUNTIFS('Fatores Externos (O-A)'!$B$6:$B$16,"Ameaça",'Fatores Externos (O-A)'!P$6:P$16,"&gt;="&amp;Parâmetros!$B$5)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I14" s="36" t="n">
         <f aca="false">G14-H14</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24129,7 +24192,7 @@
       </c>
       <c r="E40" s="39" t="n">
         <f aca="false">IF(COUNT('Fatores Externos (O-A)'!$F6:$R6)=0,"",AVERAGE('Fatores Externos (O-A)'!$F6:$R6))</f>
-        <v>2.15384615384615</v>
+        <v>2.23076923076923</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24217,7 +24280,7 @@
       </c>
       <c r="E44" s="39" t="n">
         <f aca="false">IF(COUNT('Fatores Externos (O-A)'!$F10:$R10)=0,"",AVERAGE('Fatores Externos (O-A)'!$F10:$R10))</f>
-        <v>1.76923076923077</v>
+        <v>1.84615384615385</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24257,11 +24320,11 @@
       </c>
       <c r="D46" s="36" t="n">
         <f aca="false">COUNTIF('Fatores Externos (O-A)'!$F12:$R12,"&gt;="&amp;Parâmetros!$B$5)</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E46" s="39" t="n">
         <f aca="false">IF(COUNT('Fatores Externos (O-A)'!$F12:$R12)=0,"",AVERAGE('Fatores Externos (O-A)'!$F12:$R12))</f>
-        <v>1.84615384615385</v>
+        <v>1.69230769230769</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27484,7 +27547,7 @@
       </c>
       <c r="H9" s="53" t="n">
         <f aca="false">Painel!H8</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I9" s="53" t="n">
         <f aca="false">COUNT('Fatores Externos (O-A)'!J$6:J$16)</f>
@@ -27496,11 +27559,11 @@
       </c>
       <c r="K9" s="55" t="n">
         <f aca="false">IF(I9=0,"",(G9-H9)/I9)</f>
-        <v>0</v>
+        <v>0.0909090909090909</v>
       </c>
       <c r="L9" s="56" t="n">
         <f aca="false">IF(F9="","",IF(K9="",F9,(F9+K9)/2))</f>
-        <v>0.0357142857142857</v>
+        <v>0.0811688311688312</v>
       </c>
       <c r="M9" s="46" t="n">
         <f aca="false">IF(L9="","",RANK(L9,$L$5:$L$17,0))</f>
@@ -27512,7 +27575,7 @@
       </c>
       <c r="T9" s="1" t="n">
         <f aca="false">IF(L9="",-9,L9)-ROW()*0.000000001</f>
-        <v>0.0357142767142857</v>
+        <v>0.0811688221688312</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27850,7 +27913,7 @@
       </c>
       <c r="H15" s="53" t="n">
         <f aca="false">Painel!H14</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I15" s="53" t="n">
         <f aca="false">COUNT('Fatores Externos (O-A)'!P$6:P$16)</f>
@@ -27862,11 +27925,11 @@
       </c>
       <c r="K15" s="55" t="n">
         <f aca="false">IF(I15=0,"",(G15-H15)/I15)</f>
-        <v>-0.0909090909090909</v>
+        <v>0</v>
       </c>
       <c r="L15" s="56" t="n">
         <f aca="false">IF(F15="","",IF(K15="",F15,(F15+K15)/2))</f>
-        <v>-0.25974025974026</v>
+        <v>-0.214285714285714</v>
       </c>
       <c r="M15" s="46" t="n">
         <f aca="false">IF(L15="","",RANK(L15,$L$5:$L$17,0))</f>
@@ -27878,7 +27941,7 @@
       </c>
       <c r="T15" s="1" t="n">
         <f aca="false">IF(L15="",-9,L15)-ROW()*0.000000001</f>
-        <v>-0.25974027474026</v>
+        <v>-0.214285729285714</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28065,7 +28128,7 @@
       </c>
       <c r="C23" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,2),$T$5:$T$17,0))</f>
-        <v>0.0357142857142857</v>
+        <v>0.0811688311688312</v>
       </c>
       <c r="D23" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,2),$T$5:$T$17,0))</f>
@@ -28195,7 +28258,7 @@
       </c>
       <c r="C28" s="55" t="n">
         <f aca="false">INDEX($L$5:$L$17,MATCH(LARGE($T$5:$T$17,7),$T$5:$T$17,0))</f>
-        <v>-0.25974025974026</v>
+        <v>-0.214285714285714</v>
       </c>
       <c r="D28" s="54" t="n">
         <f aca="false">INDEX($E$5:$E$17,MATCH(LARGE($T$5:$T$17,7),$T$5:$T$17,0))</f>
@@ -28465,7 +28528,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -28887,6 +28950,23 @@
       </c>
       <c r="E37" s="58" t="s">
         <v>218</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="58" t="s">
+        <v>219</v>
+      </c>
+      <c r="B38" s="58" t="s">
+        <v>220</v>
+      </c>
+      <c r="C38" s="58" t="s">
+        <v>221</v>
+      </c>
+      <c r="D38" s="58" t="s">
+        <v>222</v>
+      </c>
+      <c r="E38" s="58" t="s">
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -28921,23 +29001,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="47" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B3" s="63" t="n">
         <v>0.1</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="B4" s="64" t="n">
         <v>2</v>
@@ -28945,18 +29025,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="40" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="B5" s="65" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29083,12 +29163,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29096,40 +29176,40 @@
         <v>59</v>
       </c>
       <c r="B4" s="66" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C4" s="66" t="s">
         <v>60</v>
       </c>
       <c r="D4" s="66" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="E4" s="66" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="F4" s="66" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="G4" s="66" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="H4" s="66" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="I4" s="66" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="J4" s="66" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="K4" s="66" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="L4" s="66" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="M4" s="66" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="N4" s="66" t="s">
         <v>46</v>
@@ -29199,79 +29279,79 @@
       <c r="L5" s="66"/>
       <c r="M5" s="66"/>
       <c r="N5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="O5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="P5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="Q5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="R5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="S5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="T5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="U5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="V5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="W5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="X5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="Y5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="Z5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="AA5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AB5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="AC5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AD5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="AE5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AF5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="AG5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AH5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="AI5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AJ5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="AK5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AL5" s="67" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="AM5" s="67" t="s">
         <v>102</v>
@@ -29279,28 +29359,28 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="68" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B6" s="69" t="s">
         <v>74</v>
       </c>
       <c r="C6" s="69" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D6" s="68" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F6" s="69" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="G6" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="I6" s="71" t="n">
         <v>1</v>
@@ -29419,22 +29499,22 @@
         <v>74</v>
       </c>
       <c r="C7" s="69" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D7" s="68" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F7" s="69" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="G7" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="I7" s="71" t="n">
         <v>5602.9</v>
@@ -29549,22 +29629,22 @@
         <v>74</v>
       </c>
       <c r="C8" s="69" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="D8" s="68" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F8" s="69" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="G8" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="I8" s="71" t="n">
         <v>3.79</v>
@@ -29679,20 +29759,20 @@
         <v>74</v>
       </c>
       <c r="C9" s="69" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="D9" s="68" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F9" s="69" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="G9" s="70"/>
       <c r="H9" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="I9" s="71"/>
       <c r="J9" s="71"/>
@@ -29779,20 +29859,20 @@
         <v>74</v>
       </c>
       <c r="C10" s="69" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D10" s="68" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="G10" s="70"/>
       <c r="H10" s="70" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="I10" s="71"/>
       <c r="J10" s="71"/>
@@ -29873,28 +29953,28 @@
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="75" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="B11" s="76" t="s">
         <v>76</v>
       </c>
       <c r="C11" s="76" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D11" s="75" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F11" s="76" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="G11" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H11" s="70" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="I11" s="71" t="n">
         <v>1</v>
@@ -30013,22 +30093,22 @@
         <v>76</v>
       </c>
       <c r="C12" s="76" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D12" s="75" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F12" s="76" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="G12" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="I12" s="71" t="n">
         <v>36.92</v>
@@ -30143,22 +30223,22 @@
         <v>76</v>
       </c>
       <c r="C13" s="76" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D13" s="75" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F13" s="76" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="G13" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="I13" s="71" t="n">
         <v>2956.72</v>
@@ -30267,28 +30347,28 @@
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="77" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B14" s="78" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C14" s="78" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D14" s="77" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F14" s="78" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="G14" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="I14" s="71" t="n">
         <v>1</v>
@@ -30404,25 +30484,25 @@
         <v>194</v>
       </c>
       <c r="B15" s="78" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C15" s="78" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="D15" s="77" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F15" s="78" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="G15" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="I15" s="71" t="n">
         <v>38.11</v>
@@ -30534,25 +30614,25 @@
         <v>158</v>
       </c>
       <c r="B16" s="78" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C16" s="78" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="D16" s="77" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="E16" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F16" s="78" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="G16" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="I16" s="71" t="n">
         <v>33.22</v>
@@ -30664,25 +30744,25 @@
         <v>142</v>
       </c>
       <c r="B17" s="80" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C17" s="80" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D17" s="79" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F17" s="80" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="G17" s="70" t="n">
         <v>2023</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="I17" s="71" t="n">
         <v>74620.05</v>
@@ -30794,25 +30874,25 @@
         <v>138</v>
       </c>
       <c r="B18" s="80" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C18" s="80" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="D18" s="79" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E18" s="70" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F18" s="80" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="G18" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="I18" s="71" t="n">
         <v>11.89</v>
@@ -30924,25 +31004,25 @@
         <v>199</v>
       </c>
       <c r="B19" s="80" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C19" s="80" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D19" s="79" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="E19" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F19" s="80" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="G19" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="I19" s="71" t="n">
         <v>31.51</v>
@@ -31054,25 +31134,25 @@
         <v>202</v>
       </c>
       <c r="B20" s="80" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C20" s="80" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="D20" s="79" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E20" s="70" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F20" s="80" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="G20" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="I20" s="83" t="n">
         <v>0.1254</v>
@@ -31184,25 +31264,25 @@
         <v>160</v>
       </c>
       <c r="B21" s="80" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C21" s="80" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="D21" s="79" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E21" s="70" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F21" s="80" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="G21" s="70" t="n">
         <v>2022</v>
       </c>
       <c r="H21" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="I21" s="71" t="n">
         <v>18.24</v>
@@ -31311,7 +31391,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="33" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -31393,12 +31473,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31409,13 +31489,13 @@
         <v>67</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="D4" s="84" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="84" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="F4" s="84" t="s">
         <v>46</v>
@@ -31459,24 +31539,24 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C6" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="F6" s="70" t="n">
         <v>1</v>
@@ -31500,7 +31580,7 @@
         <v>2</v>
       </c>
       <c r="M6" s="70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N6" s="70" t="n">
         <v>2</v>
@@ -31520,19 +31600,19 @@
     </row>
     <row r="7" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C7" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="F7" s="70" t="n">
         <v>3</v>
@@ -31576,19 +31656,19 @@
     </row>
     <row r="8" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="F8" s="70" t="n">
         <v>3</v>
@@ -31632,19 +31712,19 @@
     </row>
     <row r="9" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C9" s="28" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="F9" s="70" t="n">
         <v>0</v>
@@ -31688,19 +31768,19 @@
     </row>
     <row r="10" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="F10" s="70" t="n">
         <v>1</v>
@@ -31739,24 +31819,24 @@
         <v>3</v>
       </c>
       <c r="R10" s="70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F11" s="70" t="n">
         <v>2</v>
@@ -31800,19 +31880,19 @@
     </row>
     <row r="12" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="85" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="B12" s="85" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C12" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D12" s="86" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="E12" s="86" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F12" s="70" t="n">
         <v>3</v>
@@ -31827,7 +31907,7 @@
         <v>1</v>
       </c>
       <c r="J12" s="70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" s="70" t="n">
         <v>1</v>
@@ -31845,7 +31925,7 @@
         <v>3</v>
       </c>
       <c r="P12" s="70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="70" t="n">
         <v>1</v>
@@ -31856,19 +31936,19 @@
     </row>
     <row r="13" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="85" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="B13" s="85" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C13" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D13" s="86" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="E13" s="86" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="F13" s="70" t="n">
         <v>2</v>
@@ -31912,19 +31992,19 @@
     </row>
     <row r="14" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="85" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B14" s="85" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C14" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D14" s="86" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="E14" s="86" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="F14" s="70" t="n">
         <v>3</v>
@@ -31968,19 +32048,19 @@
     </row>
     <row r="15" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="85" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="B15" s="85" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C15" s="86" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D15" s="86" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="E15" s="86" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="F15" s="70" t="n">
         <v>1</v>
@@ -32024,19 +32104,19 @@
     </row>
     <row r="16" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="85" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B16" s="85" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C16" s="86" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="D16" s="86" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="E16" s="86" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="F16" s="70" t="n">
         <v>3</v>
@@ -32080,7 +32160,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Registra áreas protegidas como evidência do OP-03 e mostra na página
- d2_ig_ativos.csv: UCs e TIs por município confirmam as notas do OP-03;
  flag de IG só repete o recorte do grupo e não foi usada.
- Página: quadro de áreas protegidas no contexto ambiental.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLDtP5x9bnGnFC43EPUEKq
</commit_message>
<xml_diff>
--- a/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
+++ b/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
@@ -413,7 +413,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="357">
   <si>
     <t xml:space="preserve">MATRIZ SWOT DO PERFIL ECONÔMICO-PRODUTIVO SETORIAL MUNICIPAL (PESM) — PANTANAL NORTE</t>
   </si>
@@ -1087,6 +1087,21 @@
     <t xml:space="preserve">Série de focos de 2023–2024 com quebra de escala (total de MT passa de ~30 mil para 0,7–1,7 milhão/ano): usar só para comparar municípios dentro do mesmo ano. d5_energia.csv mostra consumo industrial alto em Poconé (46%) e N. Sra. do Livramento (43%), ligado à mineração de ouro, não à agroindústria.</t>
   </si>
   <si>
+    <t xml:space="preserve">OP-03 (conferência)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d2_ig_ativos.csv (UCs e TIs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área de unidades de conservação e terras indígenas por município, usada como evidência do OP-03. Notas mantidas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A coluna flag_cobertura_ig_pantanal é verdadeira para os 13 municípios e falsa para os demais: só repete o recorte do grupo e não foi usada.</t>
+  </si>
+  <si>
     <t xml:space="preserve">PARÂMETROS</t>
   </si>
   <si>
@@ -1318,7 +1333,7 @@
     <t xml:space="preserve">Expansão do turismo de natureza, pesca esportiva e ecoturismo</t>
   </si>
   <si>
-    <t xml:space="preserve">SEDEC-MT; Cadastur; pesquisa de campo. Evidências: Transpantaneira (Poconé), Festival Internacional de Pesca e hidrovia (Cáceres), pesca esportiva e pousadas no rio Cuiabá (Barão de Melgaço, Sto. Antônio do Leverger); águas termais (Juscimeira); turismo de negócios e Cidade de Pedra (Rondonópolis).</t>
+    <t xml:space="preserve">SEDEC-MT; Cadastur; pesquisa de campo. Evidências: Transpantaneira (Poconé), Festival Internacional de Pesca e hidrovia (Cáceres), pesca esportiva e pousadas no rio Cuiabá (Barão de Melgaço, Sto. Antônio do Leverger); águas termais (Juscimeira); turismo de negócios e Cidade de Pedra (Rondonópolis). | Dados (d2_ig_ativos.csv, 2019): unidades de conservação em Poconé (3 UCs, 196,7 mil ha), Cáceres (4 UCs, 117,2 mil ha), Barão de Melgaço (2 UCs, 47,4 mil ha), Porto Esperidião (32,9 mil ha) e Rondonópolis (6,4 mil ha); sem UCs em Curvelândia, Glória D'Oeste, Itiquira, Juscimeira, Lambari D'Oeste, Mirassol D'Oeste e Livramento. Confirma as notas atuais.</t>
   </si>
   <si>
     <t xml:space="preserve">OP-04</t>
@@ -2678,7 +2693,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="B2" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Indicadores (F-W)'!$A$4:$AM$4,0),"")</f>
@@ -2687,7 +2702,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="B3" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Fatores Externos (O-A)'!$A$4:$R$4,0),"")</f>
@@ -2699,7 +2714,7 @@
         <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>102</v>
@@ -2708,16 +2723,16 @@
         <v>31</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>59</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>67</v>
@@ -2726,16 +2741,16 @@
         <v>33</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3539,12 +3554,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4937,7 +4952,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -4983,12 +4998,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6381,7 +6396,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -6427,12 +6442,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7825,7 +7840,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -7871,12 +7886,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9269,7 +9284,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -9315,12 +9330,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10713,7 +10728,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -10759,12 +10774,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12157,7 +12172,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -12203,12 +12218,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13601,7 +13616,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -13647,12 +13662,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15045,7 +15060,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -15091,12 +15106,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16489,7 +16504,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -17356,12 +17371,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18754,7 +18769,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -18800,12 +18815,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20198,7 +20213,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -20244,12 +20259,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21642,7 +21657,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -21688,12 +21703,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23086,7 +23101,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -28528,7 +28543,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -28967,6 +28982,23 @@
       </c>
       <c r="E38" s="58" t="s">
         <v>223</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="58" t="s">
+        <v>224</v>
+      </c>
+      <c r="B39" s="58" t="s">
+        <v>225</v>
+      </c>
+      <c r="C39" s="58" t="s">
+        <v>226</v>
+      </c>
+      <c r="D39" s="58" t="s">
+        <v>227</v>
+      </c>
+      <c r="E39" s="58" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -29001,23 +29033,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="47" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B3" s="63" t="n">
         <v>0.1</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B4" s="64" t="n">
         <v>2</v>
@@ -29025,18 +29057,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="40" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B5" s="65" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29163,12 +29195,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29176,40 +29208,40 @@
         <v>59</v>
       </c>
       <c r="B4" s="66" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="C4" s="66" t="s">
         <v>60</v>
       </c>
       <c r="D4" s="66" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="E4" s="66" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="F4" s="66" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="G4" s="66" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="H4" s="66" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="I4" s="66" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="J4" s="66" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="K4" s="66" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="L4" s="66" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="M4" s="66" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="N4" s="66" t="s">
         <v>46</v>
@@ -29279,79 +29311,79 @@
       <c r="L5" s="66"/>
       <c r="M5" s="66"/>
       <c r="N5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="O5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="P5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="Q5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="R5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="S5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="T5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="U5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="V5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="W5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="X5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="Y5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="Z5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="AA5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AB5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="AC5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AD5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="AE5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AF5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="AG5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AH5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="AI5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AJ5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="AK5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AL5" s="67" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="AM5" s="67" t="s">
         <v>102</v>
@@ -29359,28 +29391,28 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="68" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="B6" s="69" t="s">
         <v>74</v>
       </c>
       <c r="C6" s="69" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D6" s="68" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F6" s="69" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="G6" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="I6" s="71" t="n">
         <v>1</v>
@@ -29499,22 +29531,22 @@
         <v>74</v>
       </c>
       <c r="C7" s="69" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D7" s="68" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F7" s="69" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="G7" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="I7" s="71" t="n">
         <v>5602.9</v>
@@ -29629,22 +29661,22 @@
         <v>74</v>
       </c>
       <c r="C8" s="69" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D8" s="68" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F8" s="69" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="G8" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="I8" s="71" t="n">
         <v>3.79</v>
@@ -29759,20 +29791,20 @@
         <v>74</v>
       </c>
       <c r="C9" s="69" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D9" s="68" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F9" s="69" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="G9" s="70"/>
       <c r="H9" s="70" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="I9" s="71"/>
       <c r="J9" s="71"/>
@@ -29859,20 +29891,20 @@
         <v>74</v>
       </c>
       <c r="C10" s="69" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D10" s="68" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="G10" s="70"/>
       <c r="H10" s="70" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="I10" s="71"/>
       <c r="J10" s="71"/>
@@ -29953,28 +29985,28 @@
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="75" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="B11" s="76" t="s">
         <v>76</v>
       </c>
       <c r="C11" s="76" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D11" s="75" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F11" s="76" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="G11" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H11" s="70" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="I11" s="71" t="n">
         <v>1</v>
@@ -30093,22 +30125,22 @@
         <v>76</v>
       </c>
       <c r="C12" s="76" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="D12" s="75" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F12" s="76" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="G12" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="I12" s="71" t="n">
         <v>36.92</v>
@@ -30223,22 +30255,22 @@
         <v>76</v>
       </c>
       <c r="C13" s="76" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="D13" s="75" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F13" s="76" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="G13" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="I13" s="71" t="n">
         <v>2956.72</v>
@@ -30347,28 +30379,28 @@
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="77" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B14" s="78" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C14" s="78" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D14" s="77" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F14" s="78" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="G14" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="I14" s="71" t="n">
         <v>1</v>
@@ -30484,25 +30516,25 @@
         <v>194</v>
       </c>
       <c r="B15" s="78" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C15" s="78" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D15" s="77" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F15" s="78" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="G15" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="I15" s="71" t="n">
         <v>38.11</v>
@@ -30614,25 +30646,25 @@
         <v>158</v>
       </c>
       <c r="B16" s="78" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C16" s="78" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="D16" s="77" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="E16" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F16" s="78" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G16" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="I16" s="71" t="n">
         <v>33.22</v>
@@ -30744,25 +30776,25 @@
         <v>142</v>
       </c>
       <c r="B17" s="80" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C17" s="80" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="D17" s="79" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F17" s="80" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="G17" s="70" t="n">
         <v>2023</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="I17" s="71" t="n">
         <v>74620.05</v>
@@ -30874,25 +30906,25 @@
         <v>138</v>
       </c>
       <c r="B18" s="80" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C18" s="80" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="D18" s="79" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E18" s="70" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="F18" s="80" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="G18" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="I18" s="71" t="n">
         <v>11.89</v>
@@ -31004,25 +31036,25 @@
         <v>199</v>
       </c>
       <c r="B19" s="80" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C19" s="80" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="D19" s="79" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="E19" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F19" s="80" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="G19" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="I19" s="71" t="n">
         <v>31.51</v>
@@ -31134,25 +31166,25 @@
         <v>202</v>
       </c>
       <c r="B20" s="80" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C20" s="80" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D20" s="79" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="E20" s="70" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="F20" s="80" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="G20" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="I20" s="83" t="n">
         <v>0.1254</v>
@@ -31264,25 +31296,25 @@
         <v>160</v>
       </c>
       <c r="B21" s="80" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C21" s="80" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="D21" s="79" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E21" s="70" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F21" s="80" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="G21" s="70" t="n">
         <v>2022</v>
       </c>
       <c r="H21" s="70" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="I21" s="71" t="n">
         <v>18.24</v>
@@ -31391,7 +31423,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="33" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -31473,12 +31505,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31489,13 +31521,13 @@
         <v>67</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D4" s="84" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="84" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="F4" s="84" t="s">
         <v>46</v>
@@ -31539,24 +31571,24 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C6" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="F6" s="70" t="n">
         <v>1</v>
@@ -31600,19 +31632,19 @@
     </row>
     <row r="7" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C7" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F7" s="70" t="n">
         <v>3</v>
@@ -31656,19 +31688,19 @@
     </row>
     <row r="8" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="F8" s="70" t="n">
         <v>3</v>
@@ -31712,19 +31744,19 @@
     </row>
     <row r="9" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C9" s="28" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="F9" s="70" t="n">
         <v>0</v>
@@ -31768,19 +31800,19 @@
     </row>
     <row r="10" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="F10" s="70" t="n">
         <v>1</v>
@@ -31824,19 +31856,19 @@
     </row>
     <row r="11" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="F11" s="70" t="n">
         <v>2</v>
@@ -31880,19 +31912,19 @@
     </row>
     <row r="12" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="85" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B12" s="85" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C12" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D12" s="86" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="E12" s="86" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="F12" s="70" t="n">
         <v>3</v>
@@ -31936,19 +31968,19 @@
     </row>
     <row r="13" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="85" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B13" s="85" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C13" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D13" s="86" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="E13" s="86" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="F13" s="70" t="n">
         <v>2</v>
@@ -31992,19 +32024,19 @@
     </row>
     <row r="14" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="85" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="B14" s="85" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C14" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D14" s="86" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="E14" s="86" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="F14" s="70" t="n">
         <v>3</v>
@@ -32048,19 +32080,19 @@
     </row>
     <row r="15" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="85" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="B15" s="85" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C15" s="86" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D15" s="86" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="E15" s="86" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="F15" s="70" t="n">
         <v>1</v>
@@ -32104,19 +32136,19 @@
     </row>
     <row r="16" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="85" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B16" s="85" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C16" s="86" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D16" s="86" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="E16" s="86" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="F16" s="70" t="n">
         <v>3</v>
@@ -32160,7 +32192,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adiciona uso da terra ao contexto ambiental e registra perda de água no AM-01
- d4_uso_terra.csv (MapBiomas 2000-2021): gráfico de vegetação natural,
  agropecuária, água e área urbana, e quadro da variação da superfície
  de água. Queda de 63% em Cáceres, 46% em Sto. Antônio do Leverger e
  40% em Poconé registrada como evidência do AM-01 (notas mantidas).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLDtP5x9bnGnFC43EPUEKq
</commit_message>
<xml_diff>
--- a/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
+++ b/pesm-pantanal-norte/dados/Matriz_SWOT_PESM_Pantanal_Norte.xlsx
@@ -413,7 +413,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="362">
   <si>
     <t xml:space="preserve">MATRIZ SWOT DO PERFIL ECONÔMICO-PRODUTIVO SETORIAL MUNICIPAL (PESM) — PANTANAL NORTE</t>
   </si>
@@ -1102,6 +1102,21 @@
     <t xml:space="preserve">A coluna flag_cobertura_ig_pantanal é verdadeira para os 13 municípios e falsa para os demais: só repete o recorte do grupo e não foi usada.</t>
   </si>
   <si>
+    <t xml:space="preserve">AM-01 (conferência)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2000–2021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d4_uso_terra.csv (MapBiomas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variação da superfície de água por município, usada como evidência de seca prolongada. Notas mantidas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recebidos também d4_painel_pam.csv (mesmos dados de desmatamento e focos, inclusive a quebra de 2023) e novas cópias idênticas de d1_painel_pesm, d3_painel_psdm e d5_painel_pim.</t>
+  </si>
+  <si>
     <t xml:space="preserve">PARÂMETROS</t>
   </si>
   <si>
@@ -1372,7 +1387,7 @@
     <t xml:space="preserve">Eventos climáticos extremos: secas prolongadas e incêndios no Pantanal</t>
   </si>
   <si>
-    <t xml:space="preserve">INPE – BDQueimadas; MapBiomas; Cemaden. Evidências: incêndios de 2024 – Cáceres ≈87 mil ha, Poconé ≈61,5 mil ha, Barão de Melgaço ≈2,6 mil ha (Bombeiros-MT/INPE); 2020 foi o pior ano da série no Pantanal; ≈95% dos focos de 2024 começaram em propriedades privadas. Planície pantaneira = exposição alta. | Dados (d4_queimadas.csv, 2013–2022; a série de 2023–2024 muda de escala e não foi usada): focos por mil km²/ano — Barão de Melgaço 64,5; Poconé 51,4; Sto. Antônio do Leverger 34,1; N. Sra. do Livramento 30,7; Cáceres 25,4; MT 30,9; demais abaixo de 17.</t>
+    <t xml:space="preserve">INPE – BDQueimadas; MapBiomas; Cemaden. Evidências: incêndios de 2024 – Cáceres ≈87 mil ha, Poconé ≈61,5 mil ha, Barão de Melgaço ≈2,6 mil ha (Bombeiros-MT/INPE); 2020 foi o pior ano da série no Pantanal; ≈95% dos focos de 2024 começaram em propriedades privadas. Planície pantaneira = exposição alta. | Dados (d4_queimadas.csv, 2013–2022; a série de 2023–2024 muda de escala e não foi usada): focos por mil km²/ano — Barão de Melgaço 64,5; Poconé 51,4; Sto. Antônio do Leverger 34,1; N. Sra. do Livramento 30,7; Cáceres 25,4; MT 30,9; demais abaixo de 17. | Dados (d4_uso_terra.csv, MapBiomas 2000–2021): superfície de água caiu 63% em Cáceres (3.335 → 1.245 km²), 46% em Sto. Antônio do Leverger, 40% em Poconé e 13% em Barão de Melgaço; MT −29%. Confirma as notas atuais.</t>
   </si>
   <si>
     <t xml:space="preserve">AM-02</t>
@@ -2693,7 +2708,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="B2" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Indicadores (F-W)'!$A$4:$AM$4,0),"")</f>
@@ -2702,7 +2717,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="B3" s="1" t="n">
         <f aca="false">IFERROR(MATCH($B$1,'Fatores Externos (O-A)'!$A$4:$R$4,0),"")</f>
@@ -2714,7 +2729,7 @@
         <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>102</v>
@@ -2723,16 +2738,16 @@
         <v>31</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>59</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>67</v>
@@ -2741,16 +2756,16 @@
         <v>33</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3554,12 +3569,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4952,7 +4967,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -4998,12 +5013,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6396,7 +6411,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -6442,12 +6457,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7840,7 +7855,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -7886,12 +7901,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9284,7 +9299,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -9330,12 +9345,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10728,7 +10743,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -10774,12 +10789,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12172,7 +12187,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -12218,12 +12233,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13616,7 +13631,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -13662,12 +13677,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15060,7 +15075,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -15106,12 +15121,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16504,7 +16519,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -17371,12 +17386,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18769,7 +18784,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -18815,12 +18830,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20213,7 +20228,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -20259,12 +20274,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21657,7 +21672,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -21703,12 +21718,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="91" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23101,7 +23116,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="33" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -28543,7 +28558,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -28999,6 +29014,23 @@
       </c>
       <c r="E39" s="58" t="s">
         <v>228</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="58" t="s">
+        <v>229</v>
+      </c>
+      <c r="B40" s="58" t="s">
+        <v>230</v>
+      </c>
+      <c r="C40" s="58" t="s">
+        <v>231</v>
+      </c>
+      <c r="D40" s="58" t="s">
+        <v>232</v>
+      </c>
+      <c r="E40" s="58" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -29033,23 +29065,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="47" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B3" s="63" t="n">
         <v>0.1</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B4" s="64" t="n">
         <v>2</v>
@@ -29057,18 +29089,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="40" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="B5" s="65" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29195,12 +29227,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29208,40 +29240,40 @@
         <v>59</v>
       </c>
       <c r="B4" s="66" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="C4" s="66" t="s">
         <v>60</v>
       </c>
       <c r="D4" s="66" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="E4" s="66" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="F4" s="66" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="G4" s="66" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="H4" s="66" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="I4" s="66" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="J4" s="66" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="K4" s="66" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="L4" s="66" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="M4" s="66" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="N4" s="66" t="s">
         <v>46</v>
@@ -29311,79 +29343,79 @@
       <c r="L5" s="66"/>
       <c r="M5" s="66"/>
       <c r="N5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="O5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="P5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="Q5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="R5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="S5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="T5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="U5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="V5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="W5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="X5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="Y5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="Z5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="AA5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AB5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="AC5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AD5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="AE5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AF5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="AG5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AH5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="AI5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AJ5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="AK5" s="67" t="s">
         <v>102</v>
       </c>
       <c r="AL5" s="67" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="AM5" s="67" t="s">
         <v>102</v>
@@ -29391,28 +29423,28 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="68" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B6" s="69" t="s">
         <v>74</v>
       </c>
       <c r="C6" s="69" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D6" s="68" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F6" s="69" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="G6" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="I6" s="71" t="n">
         <v>1</v>
@@ -29531,22 +29563,22 @@
         <v>74</v>
       </c>
       <c r="C7" s="69" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D7" s="68" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F7" s="69" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="G7" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="I7" s="71" t="n">
         <v>5602.9</v>
@@ -29661,22 +29693,22 @@
         <v>74</v>
       </c>
       <c r="C8" s="69" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D8" s="68" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F8" s="69" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="G8" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="I8" s="71" t="n">
         <v>3.79</v>
@@ -29791,20 +29823,20 @@
         <v>74</v>
       </c>
       <c r="C9" s="69" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="D9" s="68" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F9" s="69" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="G9" s="70"/>
       <c r="H9" s="70" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="I9" s="71"/>
       <c r="J9" s="71"/>
@@ -29891,20 +29923,20 @@
         <v>74</v>
       </c>
       <c r="C10" s="69" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="D10" s="68" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="G10" s="70"/>
       <c r="H10" s="70" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="I10" s="71"/>
       <c r="J10" s="71"/>
@@ -29985,28 +30017,28 @@
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="75" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B11" s="76" t="s">
         <v>76</v>
       </c>
       <c r="C11" s="76" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="D11" s="75" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F11" s="76" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="G11" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H11" s="70" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="I11" s="71" t="n">
         <v>1</v>
@@ -30125,22 +30157,22 @@
         <v>76</v>
       </c>
       <c r="C12" s="76" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D12" s="75" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F12" s="76" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="G12" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="I12" s="71" t="n">
         <v>36.92</v>
@@ -30255,22 +30287,22 @@
         <v>76</v>
       </c>
       <c r="C13" s="76" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D13" s="75" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F13" s="76" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="G13" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="I13" s="71" t="n">
         <v>2956.72</v>
@@ -30379,28 +30411,28 @@
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="77" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="B14" s="78" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C14" s="78" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D14" s="77" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F14" s="78" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="G14" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="I14" s="71" t="n">
         <v>1</v>
@@ -30516,25 +30548,25 @@
         <v>194</v>
       </c>
       <c r="B15" s="78" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C15" s="78" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="D15" s="77" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F15" s="78" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="G15" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="I15" s="71" t="n">
         <v>38.11</v>
@@ -30646,25 +30678,25 @@
         <v>158</v>
       </c>
       <c r="B16" s="78" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C16" s="78" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="D16" s="77" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="E16" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F16" s="78" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="G16" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="I16" s="71" t="n">
         <v>33.22</v>
@@ -30776,25 +30808,25 @@
         <v>142</v>
       </c>
       <c r="B17" s="80" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C17" s="80" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="D17" s="79" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F17" s="80" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="G17" s="70" t="n">
         <v>2023</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="I17" s="71" t="n">
         <v>74620.05</v>
@@ -30906,25 +30938,25 @@
         <v>138</v>
       </c>
       <c r="B18" s="80" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C18" s="80" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D18" s="79" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E18" s="70" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="F18" s="80" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="G18" s="70" t="n">
         <v>2021</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="I18" s="71" t="n">
         <v>11.89</v>
@@ -31036,25 +31068,25 @@
         <v>199</v>
       </c>
       <c r="B19" s="80" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C19" s="80" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="D19" s="79" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="E19" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F19" s="80" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="G19" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="I19" s="71" t="n">
         <v>31.51</v>
@@ -31166,25 +31198,25 @@
         <v>202</v>
       </c>
       <c r="B20" s="80" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C20" s="80" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="D20" s="79" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="E20" s="70" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="F20" s="80" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="G20" s="70" t="n">
         <v>2024</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="I20" s="83" t="n">
         <v>0.1254</v>
@@ -31296,25 +31328,25 @@
         <v>160</v>
       </c>
       <c r="B21" s="80" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C21" s="80" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D21" s="79" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E21" s="70" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F21" s="80" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="G21" s="70" t="n">
         <v>2022</v>
       </c>
       <c r="H21" s="70" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="I21" s="71" t="n">
         <v>18.24</v>
@@ -31423,7 +31455,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="33" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -31505,12 +31537,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31521,13 +31553,13 @@
         <v>67</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="D4" s="84" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="84" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="F4" s="84" t="s">
         <v>46</v>
@@ -31571,24 +31603,24 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C6" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="F6" s="70" t="n">
         <v>1</v>
@@ -31632,19 +31664,19 @@
     </row>
     <row r="7" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C7" s="28" t="s">
         <v>74</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="F7" s="70" t="n">
         <v>3</v>
@@ -31688,19 +31720,19 @@
     </row>
     <row r="8" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="F8" s="70" t="n">
         <v>3</v>
@@ -31744,19 +31776,19 @@
     </row>
     <row r="9" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C9" s="28" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F9" s="70" t="n">
         <v>0</v>
@@ -31800,19 +31832,19 @@
     </row>
     <row r="10" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="F10" s="70" t="n">
         <v>1</v>
@@ -31856,19 +31888,19 @@
     </row>
     <row r="11" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="F11" s="70" t="n">
         <v>2</v>
@@ -31912,19 +31944,19 @@
     </row>
     <row r="12" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="85" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="B12" s="85" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C12" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D12" s="86" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="E12" s="86" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="F12" s="70" t="n">
         <v>3</v>
@@ -31968,19 +32000,19 @@
     </row>
     <row r="13" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="85" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B13" s="85" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C13" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D13" s="86" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E13" s="86" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="F13" s="70" t="n">
         <v>2</v>
@@ -32024,19 +32056,19 @@
     </row>
     <row r="14" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="85" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B14" s="85" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C14" s="86" t="s">
         <v>74</v>
       </c>
       <c r="D14" s="86" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="E14" s="86" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="F14" s="70" t="n">
         <v>3</v>
@@ -32080,19 +32112,19 @@
     </row>
     <row r="15" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="85" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="B15" s="85" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C15" s="86" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D15" s="86" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="E15" s="86" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="F15" s="70" t="n">
         <v>1</v>
@@ -32136,19 +32168,19 @@
     </row>
     <row r="16" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="85" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="B16" s="85" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C16" s="86" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D16" s="86" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E16" s="86" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="F16" s="70" t="n">
         <v>3</v>
@@ -32192,7 +32224,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>